<commit_message>
Limit feasibility comparables to Al-Qadisiyah only
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JPUqFWSAiUaUyRvwuXXupa
</commit_message>
<xml_diff>
--- a/feasibility/دراسة_جدوى_12_تاون_هاوس_القادسية.xlsx
+++ b/feasibility/دراسة_جدوى_12_تاون_هاوس_القادسية.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="250">
   <si>
     <t xml:space="preserve">فرصة استثمارية – 12 وحدة تاون هاوس | القادسية تاون هاوس (حصير) – شرق الرياض</t>
   </si>
@@ -464,10 +464,10 @@
     <t xml:space="preserve">تحقق: مجموع جدول السداد = 100%</t>
   </si>
   <si>
-    <t xml:space="preserve">المقارنات السعرية – تاون هاوس القادسية والأحياء المحيطة (شرق الرياض)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">أسعار عرض (طلب) من منصات الإعلانات – بحث بتاريخ 30 سبتمبر 2026 – مرتبة من الأغلى في القادسية. ليست صفقات منفذة.</t>
+    <t xml:space="preserve">المقارنات السعرية – تاون هاوس حي القادسية فقط (شرق الرياض)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">أسعار عرض (طلب) من منصات الإعلانات – بحث بتاريخ 30 سبتمبر 2026 – حي القادسية فقط، مرتبة من الأغلى. ليست صفقات منفذة.</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -575,78 +575,6 @@
     <t xml:space="preserve">https://www.bayut.sa/en/property/details-87578604.html</t>
   </si>
   <si>
-    <t xml:space="preserve">اليرموك</t>
-  </si>
-  <si>
-    <t xml:space="preserve">تاون هاوس فاخر 4 غرف</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://haraj.com.sa/en/11166554307/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">شقة تاون هاوس</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.propertyfinder.sa/ar/plp/للبيع/شقة-للبيع-الرياض-الرياض-اليرموك-255167.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">الرمال</t>
-  </si>
-  <si>
-    <t xml:space="preserve">تاون هاوس</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.alolayanholding.sa/properties/48919</t>
-  </si>
-  <si>
-    <t xml:space="preserve">تاون هاوس 6 غرف</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://haraj.com.sa/11146243086/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">تاون هاوس بمصعد خاص</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://haraj.com.sa/11171394967/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">تاون هاوس 5 غرف</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://dealapp.sa/ad-details/401927</t>
-  </si>
-  <si>
-    <t xml:space="preserve">الجنادرية</t>
-  </si>
-  <si>
-    <t xml:space="preserve">تاون هاوس أرضي – مخطط المعالي</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://haraj.com.sa/en/11175408706/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">مشروع تاون هاوس أرضي 3 أدوار – غصون</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.tiktok.com/@realestateprofessionals1/video/7581007983971208455</t>
-  </si>
-  <si>
-    <t xml:space="preserve">تاون هاوس أرضي – غصون</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://haraj.com.sa/en/11174873787/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">تاون هاوس – غصون</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://dwelleo.sa/ar/properties/townhouse-for-sale-in-ghsoon-al-janadriyah-east-riyadh</t>
-  </si>
-  <si>
     <t xml:space="preserve">★</t>
   </si>
   <si>
@@ -674,7 +602,7 @@
     <t xml:space="preserve">الخلايا البرتقالية في عمود السعر = وحدات أغلى من سعرنا</t>
   </si>
   <si>
-    <t xml:space="preserve">ملخص حسب الحي مقارنة بسعرنا</t>
+    <t xml:space="preserve">ملخص تاون هاوس القادسية مقارنة بسعرنا</t>
   </si>
   <si>
     <t xml:space="preserve">عدد العروض</t>
@@ -690,9 +618,6 @@
   </si>
   <si>
     <t xml:space="preserve">متوسط سعر المتر</t>
-  </si>
-  <si>
-    <t xml:space="preserve">كل المقارنات</t>
   </si>
   <si>
     <t xml:space="preserve">مشروعنا</t>
@@ -1086,7 +1011,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="52">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1263,22 +1188,6 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1292,6 +1201,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1564,11 +1477,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="26036697"/>
-        <c:axId val="11504256"/>
+        <c:axId val="45375014"/>
+        <c:axId val="21518310"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="26036697"/>
+        <c:axId val="45375014"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1600,7 +1513,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11504256"/>
+        <c:crossAx val="21518310"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1608,7 +1521,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="11504256"/>
+        <c:axId val="21518310"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1650,7 +1563,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26036697"/>
+        <c:crossAx val="45375014"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1684,13 +1597,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>-354600</xdr:colOff>
-      <xdr:row>46</xdr:row>
-      <xdr:rowOff>157320</xdr:rowOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>157680</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>61</xdr:row>
+      <xdr:row>57</xdr:row>
       <xdr:rowOff>179640</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
@@ -1699,7 +1612,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="-7733160" y="9334440"/>
+        <a:off x="-7733160" y="8572680"/>
         <a:ext cx="7199640" cy="2879640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -1968,7 +1881,7 @@
         <v>9</v>
       </c>
       <c r="F8" s="8" t="str">
-        <f aca="false">'المقارنات السعرية'!I38&amp;" من "&amp;'المقارنات السعرية'!D30</f>
+        <f aca="false">'المقارنات السعرية'!I34&amp;" من "&amp;'المقارنات السعرية'!D30</f>
         <v>7 من 7</v>
       </c>
     </row>
@@ -1977,14 +1890,14 @@
         <v>10</v>
       </c>
       <c r="C9" s="6" t="n">
-        <f aca="false">'المقارنات السعرية'!J23</f>
+        <f aca="false">'المقارنات السعرية'!J13</f>
         <v>4202.60195877796</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="9" t="n">
-        <f aca="false">'المقارنات السعرية'!I40</f>
+        <f aca="false">'المقارنات السعرية'!I36</f>
         <v>0.115384615384615</v>
       </c>
     </row>
@@ -2839,7 +2752,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:L48"/>
+  <dimension ref="B2:L44"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -3152,429 +3065,69 @@
         <v>182</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="29" t="n">
-        <v>8</v>
-      </c>
-      <c r="C13" s="29" t="s">
+    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="38" t="s">
         <v>183</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="C13" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="D13" s="16" t="s">
         <v>184</v>
       </c>
-      <c r="E13" s="29" t="s">
-        <v>178</v>
-      </c>
-      <c r="F13" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="G13" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="H13" s="33" t="n">
-        <v>251.51</v>
-      </c>
-      <c r="I13" s="34" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="J13" s="35" t="n">
-        <f aca="false">IFERROR(I13/H13,0)</f>
-        <v>7156.77309053318</v>
-      </c>
-      <c r="K13" s="29" t="s">
-        <v>163</v>
-      </c>
-      <c r="L13" s="36" t="s">
+      <c r="E13" s="38" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="29" t="n">
-        <v>9</v>
-      </c>
-      <c r="C14" s="29" t="s">
-        <v>183</v>
-      </c>
-      <c r="D14" s="4" t="s">
+      <c r="F13" s="38" t="s">
         <v>186</v>
       </c>
-      <c r="E14" s="29" t="s">
-        <v>178</v>
-      </c>
-      <c r="F14" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="G14" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="H14" s="33" t="n">
-        <v>253.5</v>
-      </c>
-      <c r="I14" s="34" t="n">
-        <v>1550000</v>
-      </c>
-      <c r="J14" s="35" t="n">
-        <f aca="false">IFERROR(I14/H14,0)</f>
-        <v>6114.39842209073</v>
-      </c>
-      <c r="K14" s="29" t="s">
-        <v>163</v>
-      </c>
-      <c r="L14" s="36" t="s">
+      <c r="G13" s="38" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="29" t="n">
-        <v>10</v>
-      </c>
-      <c r="C15" s="29" t="s">
-        <v>188</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="E15" s="29" t="s">
-        <v>178</v>
-      </c>
-      <c r="F15" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="G15" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="H15" s="33" t="n">
-        <v>260</v>
-      </c>
-      <c r="I15" s="34" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="J15" s="35" t="n">
-        <f aca="false">IFERROR(I15/H15,0)</f>
-        <v>5769.23076923077</v>
-      </c>
-      <c r="K15" s="29" t="s">
-        <v>163</v>
-      </c>
-      <c r="L15" s="36" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="29" t="n">
-        <v>11</v>
-      </c>
-      <c r="C16" s="29" t="s">
-        <v>188</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="E16" s="29" t="s">
-        <v>178</v>
-      </c>
-      <c r="F16" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="G16" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="H16" s="33" t="n">
-        <v>180</v>
-      </c>
-      <c r="I16" s="34" t="n">
-        <v>1150000</v>
-      </c>
-      <c r="J16" s="35" t="n">
-        <f aca="false">IFERROR(I16/H16,0)</f>
-        <v>6388.88888888889</v>
-      </c>
-      <c r="K16" s="29" t="s">
-        <v>163</v>
-      </c>
-      <c r="L16" s="36" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="29" t="n">
-        <v>12</v>
-      </c>
-      <c r="C17" s="29" t="s">
-        <v>188</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="E17" s="29" t="s">
-        <v>168</v>
-      </c>
-      <c r="F17" s="37" t="s">
-        <v>59</v>
-      </c>
-      <c r="G17" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="H17" s="33" t="n">
-        <v>220</v>
-      </c>
-      <c r="I17" s="34" t="n">
-        <v>1100000</v>
-      </c>
-      <c r="J17" s="35" t="n">
-        <f aca="false">IFERROR(I17/H17,0)</f>
-        <v>5000</v>
-      </c>
-      <c r="K17" s="29" t="s">
-        <v>163</v>
-      </c>
-      <c r="L17" s="36" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="29" t="n">
-        <v>13</v>
-      </c>
-      <c r="C18" s="29" t="s">
-        <v>188</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="E18" s="29" t="s">
-        <v>178</v>
-      </c>
-      <c r="F18" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="G18" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="H18" s="33" t="n">
-        <v>163.64</v>
-      </c>
-      <c r="I18" s="34" t="n">
-        <v>920000</v>
-      </c>
-      <c r="J18" s="35" t="n">
-        <f aca="false">IFERROR(I18/H18,0)</f>
-        <v>5622.09728672696</v>
-      </c>
-      <c r="K18" s="29" t="s">
-        <v>163</v>
-      </c>
-      <c r="L18" s="36" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="29" t="n">
-        <v>14</v>
-      </c>
-      <c r="C19" s="29" t="s">
-        <v>197</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="E19" s="29" t="s">
-        <v>160</v>
-      </c>
-      <c r="F19" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="G19" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="H19" s="33" t="n">
-        <v>257</v>
-      </c>
-      <c r="I19" s="34" t="n">
-        <v>1250000</v>
-      </c>
-      <c r="J19" s="35" t="n">
-        <f aca="false">IFERROR(I19/H19,0)</f>
-        <v>4863.81322957198</v>
-      </c>
-      <c r="K19" s="29" t="s">
-        <v>163</v>
-      </c>
-      <c r="L19" s="36" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="29" t="n">
-        <v>15</v>
-      </c>
-      <c r="C20" s="29" t="s">
-        <v>197</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="E20" s="29" t="s">
-        <v>160</v>
-      </c>
-      <c r="F20" s="31" t="s">
-        <v>169</v>
-      </c>
-      <c r="G20" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="H20" s="33" t="n">
-        <v>288</v>
-      </c>
-      <c r="I20" s="34" t="n">
-        <v>1080000</v>
-      </c>
-      <c r="J20" s="35" t="n">
-        <f aca="false">IFERROR(I20/H20,0)</f>
-        <v>3750</v>
-      </c>
-      <c r="K20" s="29" t="s">
-        <v>201</v>
-      </c>
-      <c r="L20" s="36" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="29" t="n">
-        <v>16</v>
-      </c>
-      <c r="C21" s="29" t="s">
-        <v>197</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="E21" s="29" t="s">
-        <v>160</v>
-      </c>
-      <c r="F21" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="G21" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="H21" s="33" t="n">
-        <v>260</v>
-      </c>
-      <c r="I21" s="34" t="n">
-        <v>900000</v>
-      </c>
-      <c r="J21" s="35" t="n">
-        <f aca="false">IFERROR(I21/H21,0)</f>
-        <v>3461.53846153846</v>
-      </c>
-      <c r="K21" s="29" t="s">
-        <v>163</v>
-      </c>
-      <c r="L21" s="36" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="29" t="n">
-        <v>17</v>
-      </c>
-      <c r="C22" s="29" t="s">
-        <v>197</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="E22" s="29" t="s">
-        <v>178</v>
-      </c>
-      <c r="F22" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="G22" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="H22" s="33" t="n">
-        <v>236.97</v>
-      </c>
-      <c r="I22" s="34" t="n">
-        <v>850000</v>
-      </c>
-      <c r="J22" s="35" t="n">
-        <f aca="false">IFERROR(I22/H22,0)</f>
-        <v>3586.95193484407</v>
-      </c>
-      <c r="K22" s="29" t="s">
-        <v>163</v>
-      </c>
-      <c r="L22" s="36" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="38" t="s">
-        <v>207</v>
-      </c>
-      <c r="C23" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="D23" s="16" t="s">
-        <v>208</v>
-      </c>
-      <c r="E23" s="38" t="s">
-        <v>209</v>
-      </c>
-      <c r="F23" s="38" t="s">
-        <v>210</v>
-      </c>
-      <c r="G23" s="38" t="s">
-        <v>211</v>
-      </c>
-      <c r="H23" s="39" t="n">
+      <c r="H13" s="39" t="n">
         <f aca="false">الافتراضات!$C$13</f>
         <v>273.64</v>
       </c>
-      <c r="I23" s="11" t="n">
+      <c r="I13" s="11" t="n">
         <f aca="false">الافتراضات!$C$8</f>
         <v>1150000</v>
       </c>
-      <c r="J23" s="40" t="n">
-        <f aca="false">IFERROR(I23/H23,0)</f>
+      <c r="J13" s="40" t="n">
+        <f aca="false">IFERROR(I13/H13,0)</f>
         <v>4202.60195877796</v>
       </c>
-      <c r="K23" s="38" t="s">
-        <v>212</v>
-      </c>
-      <c r="L23" s="16" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D24" s="41" t="s">
-        <v>214</v>
-      </c>
-      <c r="H24" s="39" t="n">
+      <c r="K13" s="38" t="s">
+        <v>188</v>
+      </c>
+      <c r="L13" s="16" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D14" s="41" t="s">
+        <v>190</v>
+      </c>
+      <c r="H14" s="39" t="n">
         <f aca="false">الافتراضات!$C$14</f>
         <v>202.24</v>
       </c>
-      <c r="I24" s="11" t="n">
+      <c r="I14" s="11" t="n">
         <f aca="false">الافتراضات!$C$8</f>
         <v>1150000</v>
       </c>
-      <c r="J24" s="40" t="n">
-        <f aca="false">IFERROR(I24/H24,0)</f>
+      <c r="J14" s="40" t="n">
+        <f aca="false">IFERROR(I14/H14,0)</f>
         <v>5686.31329113924</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D25" s="2" t="s">
-        <v>215</v>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D15" s="2" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="3" t="s">
-        <v>216</v>
+        <v>192</v>
       </c>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
@@ -3592,19 +3145,19 @@
         <v>149</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>217</v>
+        <v>193</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>218</v>
+        <v>194</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>219</v>
+        <v>195</v>
       </c>
       <c r="G29" s="14" t="s">
-        <v>220</v>
+        <v>196</v>
       </c>
       <c r="H29" s="14" t="s">
-        <v>221</v>
+        <v>197</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3612,318 +3165,218 @@
         <v>158</v>
       </c>
       <c r="D30" s="42" t="n">
-        <f aca="false">COUNTIF($C$6:$C$22,C30)</f>
+        <f aca="false">COUNTIF($C$6:$C$12,C30)</f>
         <v>7</v>
       </c>
       <c r="E30" s="35" t="n">
-        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$22,C30,$I$6:$I$22),0)</f>
+        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$12,C30,$I$6:$I$12),0)</f>
         <v>1300000</v>
       </c>
       <c r="F30" s="35" t="n">
-        <f aca="false">_xlfn.MAXIFS($I$6:$I$22,$C$6:$C$22,C30)</f>
+        <f aca="false">_xlfn.MAXIFS($I$6:$I$12,$C$6:$C$12,C30)</f>
         <v>1500000</v>
       </c>
       <c r="G30" s="43" t="n">
-        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$22,C30,$H$6:$H$22),0)</f>
+        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$12,C30,$H$6:$H$12),0)</f>
         <v>235.142857142857</v>
       </c>
       <c r="H30" s="28" t="n">
-        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$22,C30,$J$6:$J$22),0)</f>
+        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$12,C30,$J$6:$J$12),0)</f>
         <v>5575.47991239313</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C31" s="30" t="s">
-        <v>183</v>
-      </c>
-      <c r="D31" s="42" t="n">
-        <f aca="false">COUNTIF($C$6:$C$22,C31)</f>
-        <v>2</v>
-      </c>
-      <c r="E31" s="35" t="n">
-        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$22,C31,$I$6:$I$22),0)</f>
-        <v>1675000</v>
-      </c>
-      <c r="F31" s="35" t="n">
-        <f aca="false">_xlfn.MAXIFS($I$6:$I$22,$C$6:$C$22,C31)</f>
-        <v>1800000</v>
-      </c>
-      <c r="G31" s="43" t="n">
-        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$22,C31,$H$6:$H$22),0)</f>
-        <v>252.505</v>
-      </c>
-      <c r="H31" s="28" t="n">
-        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$22,C31,$J$6:$J$22),0)</f>
-        <v>6635.58575631196</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C32" s="30" t="s">
-        <v>188</v>
-      </c>
-      <c r="D32" s="42" t="n">
-        <f aca="false">COUNTIF($C$6:$C$22,C32)</f>
-        <v>4</v>
-      </c>
-      <c r="E32" s="35" t="n">
-        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$22,C32,$I$6:$I$22),0)</f>
-        <v>1167500</v>
-      </c>
-      <c r="F32" s="35" t="n">
-        <f aca="false">_xlfn.MAXIFS($I$6:$I$22,$C$6:$C$22,C32)</f>
-        <v>1500000</v>
-      </c>
-      <c r="G32" s="43" t="n">
-        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$22,C32,$H$6:$H$22),0)</f>
-        <v>205.91</v>
-      </c>
-      <c r="H32" s="28" t="n">
-        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$22,C32,$J$6:$J$22),0)</f>
-        <v>5695.05423621166</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C33" s="30" t="s">
-        <v>197</v>
-      </c>
-      <c r="D33" s="42" t="n">
-        <f aca="false">COUNTIF($C$6:$C$22,C33)</f>
-        <v>4</v>
-      </c>
-      <c r="E33" s="35" t="n">
-        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$22,C33,$I$6:$I$22),0)</f>
-        <v>1020000</v>
-      </c>
-      <c r="F33" s="35" t="n">
-        <f aca="false">_xlfn.MAXIFS($I$6:$I$22,$C$6:$C$22,C33)</f>
-        <v>1250000</v>
-      </c>
-      <c r="G33" s="43" t="n">
-        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$22,C33,$H$6:$H$22),0)</f>
-        <v>260.4925</v>
-      </c>
-      <c r="H33" s="28" t="n">
-        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$22,C33,$J$6:$J$22),0)</f>
-        <v>3915.57590648863</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C34" s="44" t="s">
-        <v>222</v>
-      </c>
-      <c r="D34" s="45" t="n">
-        <f aca="false">COUNT($I$6:$I$22)</f>
-        <v>17</v>
-      </c>
-      <c r="E34" s="46" t="n">
-        <f aca="false">AVERAGE($I$6:$I$22)</f>
-        <v>1247058.82352941</v>
-      </c>
-      <c r="F34" s="46" t="n">
-        <f aca="false">MAX($I$6:$I$22)</f>
-        <v>1800000</v>
-      </c>
-      <c r="G34" s="47" t="n">
-        <f aca="false">AVERAGE($H$6:$H$22)</f>
-        <v>236.271764705882</v>
-      </c>
-      <c r="H34" s="46" t="n">
-        <f aca="false">AVERAGE($J$6:$J$22)</f>
-        <v>5337.76773353982</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C35" s="38" t="s">
-        <v>223</v>
-      </c>
-      <c r="D35" s="48" t="n">
+      <c r="C31" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="D31" s="44" t="n">
         <f aca="false">الافتراضات!$C$7</f>
         <v>12</v>
       </c>
-      <c r="E35" s="40" t="n">
-        <f aca="false">I23</f>
+      <c r="E31" s="40" t="n">
+        <f aca="false">I13</f>
         <v>1150000</v>
       </c>
-      <c r="F35" s="40" t="n">
-        <f aca="false">I23</f>
+      <c r="F31" s="40" t="n">
+        <f aca="false">I13</f>
         <v>1150000</v>
       </c>
-      <c r="G35" s="49" t="n">
-        <f aca="false">H23</f>
+      <c r="G31" s="45" t="n">
+        <f aca="false">H13</f>
         <v>273.64</v>
       </c>
-      <c r="H35" s="40" t="n">
-        <f aca="false">J23</f>
+      <c r="H31" s="40" t="n">
+        <f aca="false">J13</f>
         <v>4202.60195877796</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="C37" s="3"/>
-      <c r="D37" s="3"/>
-      <c r="E37" s="3"/>
-      <c r="F37" s="3"/>
-      <c r="G37" s="3"/>
-      <c r="H37" s="3"/>
-      <c r="I37" s="3"/>
-      <c r="J37" s="3"/>
-      <c r="K37" s="3"/>
-      <c r="L37" s="3"/>
+    <row r="33" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="3"/>
+      <c r="K33" s="3"/>
+      <c r="L33" s="3"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C34" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="D34" s="15"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15"/>
+      <c r="H34" s="15"/>
+      <c r="I34" s="46" t="n">
+        <f aca="false">COUNTIFS($C$6:$C$12,"القادسية",$I$6:$I$12,"&gt;"&amp;I13)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C35" s="15" t="s">
+        <v>201</v>
+      </c>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+      <c r="H35" s="15"/>
+      <c r="I35" s="40" t="n">
+        <f aca="false">E30-E31</f>
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C36" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="15"/>
+      <c r="H36" s="15"/>
+      <c r="I36" s="47" t="n">
+        <f aca="false">IFERROR(1-E31/E30,0)</f>
+        <v>0.115384615384615</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C37" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="D37" s="15"/>
+      <c r="E37" s="15"/>
+      <c r="F37" s="15"/>
+      <c r="G37" s="15"/>
+      <c r="H37" s="15"/>
+      <c r="I37" s="47" t="n">
+        <f aca="false">IFERROR(1-E31/F30,0)</f>
+        <v>0.233333333333333</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C38" s="15" t="s">
-        <v>225</v>
+        <v>204</v>
       </c>
       <c r="D38" s="15"/>
       <c r="E38" s="15"/>
       <c r="F38" s="15"/>
       <c r="G38" s="15"/>
       <c r="H38" s="15"/>
-      <c r="I38" s="50" t="n">
-        <f aca="false">COUNTIFS($C$6:$C$22,"القادسية",$I$6:$I$22,"&gt;"&amp;I23)</f>
-        <v>7</v>
+      <c r="I38" s="45" t="n">
+        <f aca="false">G31-G30</f>
+        <v>38.4971428571429</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C39" s="15" t="s">
-        <v>226</v>
+        <v>205</v>
       </c>
       <c r="D39" s="15"/>
       <c r="E39" s="15"/>
       <c r="F39" s="15"/>
       <c r="G39" s="15"/>
       <c r="H39" s="15"/>
-      <c r="I39" s="40" t="n">
-        <f aca="false">E30-E35</f>
-        <v>150000</v>
+      <c r="I39" s="47" t="n">
+        <f aca="false">IFERROR(1-H31/H30,0)</f>
+        <v>0.246234938550052</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C40" s="15" t="s">
-        <v>227</v>
+        <v>206</v>
       </c>
       <c r="D40" s="15"/>
       <c r="E40" s="15"/>
       <c r="F40" s="15"/>
       <c r="G40" s="15"/>
       <c r="H40" s="15"/>
-      <c r="I40" s="51" t="n">
-        <f aca="false">IFERROR(1-E35/E30,0)</f>
-        <v>0.115384615384615</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C41" s="15" t="s">
-        <v>228</v>
-      </c>
-      <c r="D41" s="15"/>
-      <c r="E41" s="15"/>
-      <c r="F41" s="15"/>
-      <c r="G41" s="15"/>
-      <c r="H41" s="15"/>
-      <c r="I41" s="51" t="n">
-        <f aca="false">IFERROR(1-E35/F30,0)</f>
-        <v>0.233333333333333</v>
+      <c r="I40" s="47" t="n">
+        <f aca="false">IFERROR(1-J14/H30,0)</f>
+        <v>-0.019878715462637</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C42" s="15" t="s">
-        <v>229</v>
-      </c>
-      <c r="D42" s="15"/>
-      <c r="E42" s="15"/>
-      <c r="F42" s="15"/>
-      <c r="G42" s="15"/>
-      <c r="H42" s="15"/>
-      <c r="I42" s="49" t="n">
-        <f aca="false">G35-G30</f>
-        <v>38.4971428571429</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C43" s="15" t="s">
-        <v>230</v>
-      </c>
-      <c r="D43" s="15"/>
-      <c r="E43" s="15"/>
-      <c r="F43" s="15"/>
-      <c r="G43" s="15"/>
-      <c r="H43" s="15"/>
-      <c r="I43" s="51" t="n">
-        <f aca="false">IFERROR(1-H35/H30,0)</f>
-        <v>0.246234938550052</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C44" s="15" t="s">
-        <v>231</v>
-      </c>
-      <c r="D44" s="15"/>
-      <c r="E44" s="15"/>
-      <c r="F44" s="15"/>
-      <c r="G44" s="15"/>
-      <c r="H44" s="15"/>
-      <c r="I44" s="51" t="n">
-        <f aca="false">IFERROR(1-J24/H30,0)</f>
-        <v>-0.019878715462637</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C46" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="D46" s="13"/>
-      <c r="E46" s="13"/>
-      <c r="F46" s="13"/>
-      <c r="G46" s="13"/>
-      <c r="H46" s="13"/>
-      <c r="I46" s="13"/>
-      <c r="J46" s="13"/>
-      <c r="K46" s="13"/>
-      <c r="L46" s="13"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C47" s="13"/>
-      <c r="D47" s="13"/>
-      <c r="E47" s="13"/>
-      <c r="F47" s="13"/>
-      <c r="G47" s="13"/>
-      <c r="H47" s="13"/>
-      <c r="I47" s="13"/>
-      <c r="J47" s="13"/>
-      <c r="K47" s="13"/>
-      <c r="L47" s="13"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C48" s="13"/>
-      <c r="D48" s="13"/>
-      <c r="E48" s="13"/>
-      <c r="F48" s="13"/>
-      <c r="G48" s="13"/>
-      <c r="H48" s="13"/>
-      <c r="I48" s="13"/>
-      <c r="J48" s="13"/>
-      <c r="K48" s="13"/>
-      <c r="L48" s="13"/>
+      <c r="C42" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="D42" s="13"/>
+      <c r="E42" s="13"/>
+      <c r="F42" s="13"/>
+      <c r="G42" s="13"/>
+      <c r="H42" s="13"/>
+      <c r="I42" s="13"/>
+      <c r="J42" s="13"/>
+      <c r="K42" s="13"/>
+      <c r="L42" s="13"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C43" s="13"/>
+      <c r="D43" s="13"/>
+      <c r="E43" s="13"/>
+      <c r="F43" s="13"/>
+      <c r="G43" s="13"/>
+      <c r="H43" s="13"/>
+      <c r="I43" s="13"/>
+      <c r="J43" s="13"/>
+      <c r="K43" s="13"/>
+      <c r="L43" s="13"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C44" s="13"/>
+      <c r="D44" s="13"/>
+      <c r="E44" s="13"/>
+      <c r="F44" s="13"/>
+      <c r="G44" s="13"/>
+      <c r="H44" s="13"/>
+      <c r="I44" s="13"/>
+      <c r="J44" s="13"/>
+      <c r="K44" s="13"/>
+      <c r="L44" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="B28:L28"/>
-    <mergeCell ref="B37:L37"/>
+    <mergeCell ref="B33:L33"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="C35:H35"/>
+    <mergeCell ref="C36:H36"/>
+    <mergeCell ref="C37:H37"/>
     <mergeCell ref="C38:H38"/>
     <mergeCell ref="C39:H39"/>
     <mergeCell ref="C40:H40"/>
-    <mergeCell ref="C41:H41"/>
-    <mergeCell ref="C42:H42"/>
-    <mergeCell ref="C43:H43"/>
-    <mergeCell ref="C44:H44"/>
-    <mergeCell ref="C46:L48"/>
+    <mergeCell ref="C42:L44"/>
   </mergeCells>
-  <conditionalFormatting sqref="I6:I22">
+  <conditionalFormatting sqref="I6:I12">
     <cfRule type="cellIs" priority="2" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>$I$23</formula>
+      <formula>$I$13</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
@@ -3934,16 +3387,6 @@
     <hyperlink ref="L10" r:id="rId5" display="https://haraj.com.sa/en/11164555558/"/>
     <hyperlink ref="L11" r:id="rId6" display="https://haraj.com.sa/11151387860/"/>
     <hyperlink ref="L12" r:id="rId7" display="https://www.bayut.sa/en/property/details-87578604.html"/>
-    <hyperlink ref="L13" r:id="rId8" display="https://haraj.com.sa/en/11166554307/"/>
-    <hyperlink ref="L14" r:id="rId9" display="https://www.propertyfinder.sa/ar/plp/للبيع/شقة-للبيع-الرياض-الرياض-اليرموك-255167.html"/>
-    <hyperlink ref="L15" r:id="rId10" display="https://www.alolayanholding.sa/properties/48919"/>
-    <hyperlink ref="L16" r:id="rId11" display="https://haraj.com.sa/11146243086/"/>
-    <hyperlink ref="L17" r:id="rId12" display="https://haraj.com.sa/11171394967/"/>
-    <hyperlink ref="L18" r:id="rId13" display="https://dealapp.sa/ad-details/401927"/>
-    <hyperlink ref="L19" r:id="rId14" display="https://haraj.com.sa/en/11175408706/"/>
-    <hyperlink ref="L20" r:id="rId15" display="https://www.tiktok.com/@realestateprofessionals1/video/7581007983971208455"/>
-    <hyperlink ref="L21" r:id="rId16" display="https://haraj.com.sa/en/11174873787/"/>
-    <hyperlink ref="L22" r:id="rId17" display="https://dwelleo.sa/ar/properties/townhouse-for-sale-in-ghsoon-al-janadriyah-east-riyadh"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3952,7 +3395,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId18"/>
+  <drawing r:id="rId8"/>
 </worksheet>
 </file>
 
@@ -3972,12 +3415,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="21.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>233</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>234</v>
+        <v>209</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -3988,7 +3431,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
-        <v>235</v>
+        <v>210</v>
       </c>
       <c r="C5" s="35" t="n">
         <f aca="false">الافتراضات!$C$7*الافتراضات!$C$8</f>
@@ -3997,7 +3440,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
-        <v>236</v>
+        <v>211</v>
       </c>
       <c r="C6" s="35" t="n">
         <f aca="false">C5*(الافتراضات!$C$16+الافتراضات!$C$17)</f>
@@ -4006,7 +3449,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="15" t="s">
-        <v>237</v>
+        <v>212</v>
       </c>
       <c r="C7" s="28" t="n">
         <f aca="false">C5+C6</f>
@@ -4015,7 +3458,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="4" t="s">
-        <v>238</v>
+        <v>213</v>
       </c>
       <c r="C8" s="35" t="n">
         <f aca="false">الافتراضات!$C$7*الافتراضات!$C$25</f>
@@ -4024,7 +3467,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="4" t="s">
-        <v>239</v>
+        <v>214</v>
       </c>
       <c r="C9" s="35" t="n">
         <f aca="false">الافتراضات!$C$7*'المقارنات السعرية'!E30</f>
@@ -4033,7 +3476,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="15" t="s">
-        <v>240</v>
+        <v>215</v>
       </c>
       <c r="C10" s="40" t="n">
         <f aca="false">C8-C5</f>
@@ -4042,7 +3485,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
-        <v>241</v>
+        <v>216</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
@@ -4056,27 +3499,27 @@
         <v>91</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>242</v>
+        <v>217</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>243</v>
+        <v>218</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>244</v>
+        <v>219</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>245</v>
+        <v>220</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>246</v>
+        <v>221</v>
       </c>
       <c r="H13" s="14" t="s">
-        <v>247</v>
+        <v>222</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="4" t="s">
-        <v>248</v>
+        <v>223</v>
       </c>
       <c r="C14" s="35" t="n">
         <f aca="false">-الافتراضات!$C$19*$C$5</f>
@@ -4105,7 +3548,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="4" t="s">
-        <v>249</v>
+        <v>224</v>
       </c>
       <c r="C15" s="35" t="n">
         <f aca="false">IF(0=0,-$C$6,0)</f>
@@ -4134,7 +3577,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="4" t="s">
-        <v>250</v>
+        <v>225</v>
       </c>
       <c r="C16" s="35" t="n">
         <f aca="false">IF(0*0.5=ROUND(الافتراضات!$C$28,1),الافتراضات!$C$7*الافتراضات!$C$29,0)</f>
@@ -4163,7 +3606,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="4" t="s">
-        <v>251</v>
+        <v>226</v>
       </c>
       <c r="C17" s="35" t="n">
         <f aca="false">-C16*(الافتراضات!$C$30+الافتراضات!$C$31)</f>
@@ -4192,36 +3635,36 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="15" t="s">
-        <v>252</v>
-      </c>
-      <c r="C18" s="46" t="n">
+        <v>227</v>
+      </c>
+      <c r="C18" s="48" t="n">
         <f aca="false">SUM(C14:C17)</f>
         <v>-14490000</v>
       </c>
-      <c r="D18" s="46" t="n">
+      <c r="D18" s="48" t="n">
         <f aca="false">SUM(D14:D17)</f>
         <v>0</v>
       </c>
-      <c r="E18" s="46" t="n">
+      <c r="E18" s="48" t="n">
         <f aca="false">SUM(E14:E17)</f>
         <v>0</v>
       </c>
-      <c r="F18" s="46" t="n">
+      <c r="F18" s="48" t="n">
         <f aca="false">SUM(F14:F17)</f>
         <v>0</v>
       </c>
-      <c r="G18" s="46" t="n">
+      <c r="G18" s="48" t="n">
         <f aca="false">SUM(G14:G17)</f>
         <v>14985000</v>
       </c>
-      <c r="H18" s="46" t="n">
+      <c r="H18" s="48" t="n">
         <f aca="false">SUM(C18:G18)</f>
         <v>495000</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="4" t="s">
-        <v>253</v>
+        <v>228</v>
       </c>
       <c r="C19" s="35" t="n">
         <f aca="false">SUM($C$18:C18)</f>
@@ -4250,7 +3693,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
-        <v>254</v>
+        <v>229</v>
       </c>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
@@ -4261,7 +3704,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="15" t="s">
-        <v>255</v>
+        <v>230</v>
       </c>
       <c r="C22" s="40" t="n">
         <f aca="false">H18</f>
@@ -4270,34 +3713,34 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="15" t="s">
-        <v>256</v>
-      </c>
-      <c r="C23" s="51" t="n">
+        <v>231</v>
+      </c>
+      <c r="C23" s="47" t="n">
         <f aca="false">IFERROR(H18/-SUMIF(C18:G18,"&lt;0"),0)</f>
         <v>0.0341614906832298</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="15" t="s">
-        <v>257</v>
-      </c>
-      <c r="C24" s="51" t="n">
+        <v>232</v>
+      </c>
+      <c r="C24" s="47" t="n">
         <f aca="false">IFERROR(C23/الافتراضات!$C$28,0)</f>
         <v>0.0170807453416149</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="15" t="s">
-        <v>258</v>
-      </c>
-      <c r="C25" s="51" t="n">
+        <v>233</v>
+      </c>
+      <c r="C25" s="47" t="n">
         <f aca="false">IFERROR((1+IRR(C18:G18))^2-1,0)</f>
         <v>0.0169373091214771</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="15" t="s">
-        <v>259</v>
+        <v>234</v>
       </c>
       <c r="C26" s="40" t="n">
         <f aca="false">IFERROR(C7/(1-الافتراضات!$C$30-الافتراضات!$C$31)/الافتراضات!$C$7,0)</f>
@@ -4306,16 +3749,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="15" t="s">
-        <v>260</v>
-      </c>
-      <c r="C27" s="51" t="n">
+        <v>235</v>
+      </c>
+      <c r="C27" s="47" t="n">
         <f aca="false">IFERROR(1-C26/الافتراضات!$C$29,0)</f>
         <v>0.033033033033033</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="3" t="s">
-        <v>261</v>
+        <v>236</v>
       </c>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
@@ -4326,33 +3769,33 @@
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="14" t="s">
-        <v>262</v>
+        <v>237</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>263</v>
+        <v>238</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>264</v>
+        <v>239</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>265</v>
+        <v>240</v>
       </c>
       <c r="F30" s="14" t="s">
-        <v>264</v>
+        <v>239</v>
       </c>
       <c r="G30" s="14" t="s">
-        <v>266</v>
+        <v>241</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="52" t="n">
+      <c r="B31" s="49" t="n">
         <v>1200000</v>
       </c>
       <c r="C31" s="28" t="n">
         <f aca="false">الافتراضات!$C$7*B31*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)</f>
         <v>-1170000</v>
       </c>
-      <c r="D31" s="53" t="n">
+      <c r="D31" s="50" t="n">
         <f aca="false">IFERROR(C31/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)),0)</f>
         <v>-0.080745341614907</v>
       </c>
@@ -4360,24 +3803,24 @@
         <f aca="false">الافتراضات!$C$7*B31*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)</f>
         <v>-480000.000000002</v>
       </c>
-      <c r="F31" s="53" t="n">
+      <c r="F31" s="50" t="n">
         <f aca="false">IFERROR(E31/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)),0)</f>
         <v>-0.0347826086956523</v>
       </c>
-      <c r="G31" s="53" t="n">
+      <c r="G31" s="50" t="n">
         <f aca="false">IFERROR((الافتراضات!$C$7*B31*(1-الافتراضات!$C$30-الافتراضات!$C$31)/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)))^(1/الافتراضات!$C$28)-1,0)</f>
         <v>-0.0175452217509715</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="52" t="n">
+      <c r="B32" s="49" t="n">
         <v>1250000</v>
       </c>
       <c r="C32" s="28" t="n">
         <f aca="false">الافتراضات!$C$7*B32*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)</f>
         <v>-615000.000000002</v>
       </c>
-      <c r="D32" s="53" t="n">
+      <c r="D32" s="50" t="n">
         <f aca="false">IFERROR(C32/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)),0)</f>
         <v>-0.0424430641821948</v>
       </c>
@@ -4385,24 +3828,24 @@
         <f aca="false">الافتراضات!$C$7*B32*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)</f>
         <v>74999.9999999981</v>
       </c>
-      <c r="F32" s="53" t="n">
+      <c r="F32" s="50" t="n">
         <f aca="false">IFERROR(E32/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)),0)</f>
         <v>0.00543478260869552</v>
       </c>
-      <c r="G32" s="53" t="n">
+      <c r="G32" s="50" t="n">
         <f aca="false">IFERROR((الافتراضات!$C$7*B32*(1-الافتراضات!$C$30-الافتراضات!$C$31)/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)))^(1/الافتراضات!$C$28)-1,0)</f>
         <v>0.0027137091955487</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="52" t="n">
+      <c r="B33" s="49" t="n">
         <v>1300000</v>
       </c>
       <c r="C33" s="28" t="n">
         <f aca="false">الافتراضات!$C$7*B33*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)</f>
         <v>-60000.0000000019</v>
       </c>
-      <c r="D33" s="53" t="n">
+      <c r="D33" s="50" t="n">
         <f aca="false">IFERROR(C33/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)),0)</f>
         <v>-0.00414078674948253</v>
       </c>
@@ -4410,24 +3853,24 @@
         <f aca="false">الافتراضات!$C$7*B33*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)</f>
         <v>629999.999999998</v>
       </c>
-      <c r="F33" s="53" t="n">
+      <c r="F33" s="50" t="n">
         <f aca="false">IFERROR(E33/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)),0)</f>
         <v>0.0456521739130434</v>
       </c>
-      <c r="G33" s="53" t="n">
+      <c r="G33" s="50" t="n">
         <f aca="false">IFERROR((الافتراضات!$C$7*B33*(1-الافتراضات!$C$30-الافتراضات!$C$31)/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)))^(1/الافتراضات!$C$28)-1,0)</f>
         <v>0.0225713539470209</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="52" t="n">
+      <c r="B34" s="49" t="n">
         <v>1350000</v>
       </c>
       <c r="C34" s="28" t="n">
         <f aca="false">الافتراضات!$C$7*B34*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)</f>
         <v>494999.999999998</v>
       </c>
-      <c r="D34" s="53" t="n">
+      <c r="D34" s="50" t="n">
         <f aca="false">IFERROR(C34/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)),0)</f>
         <v>0.0341614906832297</v>
       </c>
@@ -4435,24 +3878,24 @@
         <f aca="false">الافتراضات!$C$7*B34*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)</f>
         <v>1185000</v>
       </c>
-      <c r="F34" s="53" t="n">
+      <c r="F34" s="50" t="n">
         <f aca="false">IFERROR(E34/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)),0)</f>
         <v>0.0858695652173912</v>
       </c>
-      <c r="G34" s="53" t="n">
+      <c r="G34" s="50" t="n">
         <f aca="false">IFERROR((الافتراضات!$C$7*B34*(1-الافتراضات!$C$30-الافتراضات!$C$31)/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)))^(1/الافتراضات!$C$28)-1,0)</f>
         <v>0.0420506538635208</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="52" t="n">
+      <c r="B35" s="49" t="n">
         <v>1400000</v>
       </c>
       <c r="C35" s="28" t="n">
         <f aca="false">الافتراضات!$C$7*B35*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)</f>
         <v>1050000</v>
       </c>
-      <c r="D35" s="53" t="n">
+      <c r="D35" s="50" t="n">
         <f aca="false">IFERROR(C35/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)),0)</f>
         <v>0.0724637681159419</v>
       </c>
@@ -4460,24 +3903,24 @@
         <f aca="false">الافتراضات!$C$7*B35*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)</f>
         <v>1740000</v>
       </c>
-      <c r="F35" s="53" t="n">
+      <c r="F35" s="50" t="n">
         <f aca="false">IFERROR(E35/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)),0)</f>
         <v>0.126086956521739</v>
       </c>
-      <c r="G35" s="53" t="n">
+      <c r="G35" s="50" t="n">
         <f aca="false">IFERROR((الافتراضات!$C$7*B35*(1-الافتراضات!$C$30-الافتراضات!$C$31)/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)))^(1/الافتراضات!$C$28)-1,0)</f>
         <v>0.0611724442906247</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="52" t="n">
+      <c r="B36" s="49" t="n">
         <v>1450000</v>
       </c>
       <c r="C36" s="28" t="n">
         <f aca="false">الافتراضات!$C$7*B36*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)</f>
         <v>1605000</v>
       </c>
-      <c r="D36" s="53" t="n">
+      <c r="D36" s="50" t="n">
         <f aca="false">IFERROR(C36/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)),0)</f>
         <v>0.110766045548654</v>
       </c>
@@ -4485,24 +3928,24 @@
         <f aca="false">الافتراضات!$C$7*B36*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)</f>
         <v>2295000</v>
       </c>
-      <c r="F36" s="53" t="n">
+      <c r="F36" s="50" t="n">
         <f aca="false">IFERROR(E36/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)),0)</f>
         <v>0.166304347826087</v>
       </c>
-      <c r="G36" s="53" t="n">
+      <c r="G36" s="50" t="n">
         <f aca="false">IFERROR((الافتراضات!$C$7*B36*(1-الافتراضات!$C$30-الافتراضات!$C$31)/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)))^(1/الافتراضات!$C$28)-1,0)</f>
         <v>0.079955715678234</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="52" t="n">
+      <c r="B37" s="49" t="n">
         <v>1500000</v>
       </c>
       <c r="C37" s="28" t="n">
         <f aca="false">الافتراضات!$C$7*B37*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)</f>
         <v>2160000</v>
       </c>
-      <c r="D37" s="53" t="n">
+      <c r="D37" s="50" t="n">
         <f aca="false">IFERROR(C37/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)),0)</f>
         <v>0.149068322981366</v>
       </c>
@@ -4510,24 +3953,24 @@
         <f aca="false">الافتراضات!$C$7*B37*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)</f>
         <v>2850000</v>
       </c>
-      <c r="F37" s="53" t="n">
+      <c r="F37" s="50" t="n">
         <f aca="false">IFERROR(E37/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)),0)</f>
         <v>0.206521739130435</v>
       </c>
-      <c r="G37" s="53" t="n">
+      <c r="G37" s="50" t="n">
         <f aca="false">IFERROR((الافتراضات!$C$7*B37*(1-الافتراضات!$C$30-الافتراضات!$C$31)/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)))^(1/الافتراضات!$C$28)-1,0)</f>
         <v>0.0984178344921547</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="52" t="n">
+      <c r="B38" s="49" t="n">
         <v>1550000</v>
       </c>
       <c r="C38" s="28" t="n">
         <f aca="false">الافتراضات!$C$7*B38*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)</f>
         <v>2715000</v>
       </c>
-      <c r="D38" s="53" t="n">
+      <c r="D38" s="50" t="n">
         <f aca="false">IFERROR(C38/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)),0)</f>
         <v>0.187370600414079</v>
       </c>
@@ -4535,23 +3978,23 @@
         <f aca="false">الافتراضات!$C$7*B38*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)</f>
         <v>3405000</v>
       </c>
-      <c r="F38" s="53" t="n">
+      <c r="F38" s="50" t="n">
         <f aca="false">IFERROR(E38/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)),0)</f>
         <v>0.246739130434783</v>
       </c>
-      <c r="G38" s="53" t="n">
+      <c r="G38" s="50" t="n">
         <f aca="false">IFERROR((الافتراضات!$C$7*B38*(1-الافتراضات!$C$30-الافتراضات!$C$31)/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)))^(1/الافتراضات!$C$28)-1,0)</f>
         <v>0.116574731236017</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="2" t="s">
-        <v>267</v>
+        <v>242</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="3" t="s">
-        <v>268</v>
+        <v>243</v>
       </c>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
@@ -4562,7 +4005,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="4" t="s">
-        <v>269</v>
+        <v>244</v>
       </c>
       <c r="C42" s="28" t="n">
         <f aca="false">الافتراضات!$C$7*الافتراضات!$C$33</f>
@@ -4571,7 +4014,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="4" t="s">
-        <v>270</v>
+        <v>245</v>
       </c>
       <c r="C43" s="28" t="n">
         <f aca="false">C42*الافتراضات!$C$34</f>
@@ -4580,7 +4023,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="15" t="s">
-        <v>271</v>
+        <v>246</v>
       </c>
       <c r="C44" s="28" t="n">
         <f aca="false">C43*(1-الافتراضات!$C$35)</f>
@@ -4589,27 +4032,27 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="C45" s="51" t="n">
+        <v>247</v>
+      </c>
+      <c r="C45" s="47" t="n">
         <f aca="false">IFERROR(C42/C5,0)</f>
         <v>0.0652173913043478</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="C46" s="51" t="n">
+        <v>248</v>
+      </c>
+      <c r="C46" s="47" t="n">
         <f aca="false">IFERROR(C44/C7,0)</f>
         <v>0.0548757763975155</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="C47" s="54" t="n">
+        <v>249</v>
+      </c>
+      <c r="C47" s="51" t="n">
         <f aca="false">IFERROR(C42/C9,0)</f>
         <v>0.0576923076923077</v>
       </c>

</xml_diff>

<commit_message>
Add higher-priced Al-Qadisiyah townhouse comps and villa price-ceiling reference
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JPUqFWSAiUaUyRvwuXXupa
</commit_message>
<xml_diff>
--- a/feasibility/دراسة_جدوى_12_تاون_هاوس_القادسية.xlsx
+++ b/feasibility/دراسة_جدوى_12_تاون_هاوس_القادسية.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="269">
   <si>
     <t xml:space="preserve">فرصة استثمارية – 12 وحدة تاون هاوس | القادسية تاون هاوس (حصير) – شرق الرياض</t>
   </si>
@@ -503,6 +503,21 @@
     <t xml:space="preserve">القادسية</t>
   </si>
   <si>
+    <t xml:space="preserve">تاون هاوس جديد لم يُسكن – 6 غرف</t>
+  </si>
+  <si>
+    <t xml:space="preserve">غير محدد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">غير مذكور</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://haraj.com.sa/11151459820/</t>
+  </si>
+  <si>
     <t xml:space="preserve">تاون هاوس أرضي على شارع 20</t>
   </si>
   <si>
@@ -512,12 +527,6 @@
     <t xml:space="preserve">للعلوي فقط</t>
   </si>
   <si>
-    <t xml:space="preserve">غير مذكور</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://haraj.com.sa/11140216303/</t>
   </si>
   <si>
@@ -539,6 +548,9 @@
     <t xml:space="preserve">https://sa.aqar.fm/فلل-للبيع/الرياض/شرق-الرياض/حي-القادسية/تاون-هاوس</t>
   </si>
   <si>
+    <t xml:space="preserve">تاون هاوس 3 أدوار بمجمع سكني – 4 دقائق من طريق الملك عبدالله (عمر سنتين)</t>
+  </si>
+  <si>
     <t xml:space="preserve">شقة تاون هاوس دوبلكس 3 أدوار</t>
   </si>
   <si>
@@ -560,9 +572,6 @@
     <t xml:space="preserve">فيلا تاون هاوس</t>
   </si>
   <si>
-    <t xml:space="preserve">غير محدد</t>
-  </si>
-  <si>
     <t xml:space="preserve">أغسطس 2025</t>
   </si>
   <si>
@@ -648,6 +657,54 @@
   </si>
   <si>
     <t xml:space="preserve">ملاحظات: (1) بعض الإعلانات تذكر مساحة الأرض وبعضها مسطح البناء. (2) "غير مذكور" = الميزة لم تُذكر في نص الإعلان. (3) مشاريع مطورين أخرى في القادسية بدون أسعار معلنة: "نجد الأول" من ريبورتاج (24 تاون هاوس) و"أملا" (14 فيلا متصلة). (4) يُنصح بالتحقق الميداني قبل العرض النهائي.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">مرجع السقف السعري – فلل مستقلة معروضة في حي القادسية (ليست تاون هاوس)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">النوع</t>
+  </si>
+  <si>
+    <t xml:space="preserve">فيلا على شارع 15 غرب – 8 غرف، ملحق وغرفة خادمة</t>
+  </si>
+  <si>
+    <t xml:space="preserve">فيلا مستقلة</t>
+  </si>
+  <si>
+    <t xml:space="preserve">✓ مركب</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.bayut.sa/en/property/details-87614706.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">فيلا في موقع قريب من الخدمات</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://sa.aqar.fm/فلل-للبيع/الرياض/شرق-الرياض/حي-القادسية</t>
+  </si>
+  <si>
+    <t xml:space="preserve">فيلا درج داخلي بدون شقق – 4 غرف (أرض 220م، مسطح 333م)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://haraj.com.sa/search/فيلا للبيع في حي القادسية في الرياض/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">فيلا 7 غرف</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.propertyfinder.sa/en/buy/ar-riyadh/villas-for-sale-al-qadisiyah.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">فيلا 5 غرف</t>
+  </si>
+  <si>
+    <t xml:space="preserve">متوسط الفلل المستقلة</t>
+  </si>
+  <si>
+    <t xml:space="preserve">سعر وحدتنا أقل من متوسط الفلل المستقلة بنسبة</t>
+  </si>
+  <si>
+    <t xml:space="preserve">الفلل للاستدلال على سقف الأسعار في الحي فقط، ولا تدخل في متوسطات التاون هاوس أعلاه.</t>
   </si>
   <si>
     <t xml:space="preserve">العائد على المستثمر – إعادة البيع بعد التسليم + التأجير</t>
@@ -895,16 +952,16 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFBF8F00"/>
+      <u val="single"/>
+      <sz val="9"/>
+      <color rgb="FF0563C1"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <u val="single"/>
-      <sz val="9"/>
-      <color rgb="FF0563C1"/>
+      <sz val="11"/>
+      <color rgb="FFBF8F00"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1011,7 +1068,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1136,10 +1193,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1156,8 +1209,12 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1201,6 +1258,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1417,28 +1482,34 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'المقارنات السعرية'!$D$6:$D$12</c:f>
+              <c:f>'المقارنات السعرية'!$D$6:$D$14</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
+                  <c:v>تاون هاوس جديد لم يُسكن – 6 غرف</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>تاون هاوس أرضي على شارع 20</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>تاون هاوس علوي – نفس المبنى</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>تاون هاوس مودرن واجهة شرقية 4 غرف</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
+                  <c:v>تاون هاوس 3 أدوار بمجمع سكني – 4 دقائق من طريق الملك عبدالله (عمر سنتين)</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>شقة تاون هاوس دوبلكس 3 أدوار</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="6">
                   <c:v>تاون هاوس علوي بمصعد وعداد مستقل</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="7">
                   <c:v>فيلا تاون هاوس</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="8">
                   <c:v>تاون هاوس – شارع 30 غرب، 3 غرف</c:v>
                 </c:pt>
               </c:strCache>
@@ -1446,29 +1517,35 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'المقارنات السعرية'!$I$6:$I$12</c:f>
+              <c:f>'المقارنات السعرية'!$I$6:$I$14</c:f>
               <c:numCache>
                 <c:formatCode>#,##0;\(#,##0\);\-</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
+                  <c:v>1550000</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>1500000</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>1400000</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>1350000</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
+                  <c:v>1300000</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>1250000</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="6">
                   <c:v>1200000</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="7">
                   <c:v>1200000</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="8">
                   <c:v>1200000</c:v>
                 </c:pt>
               </c:numCache>
@@ -1477,11 +1554,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="45375014"/>
-        <c:axId val="21518310"/>
+        <c:axId val="28970228"/>
+        <c:axId val="12868119"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="45375014"/>
+        <c:axId val="28970228"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1513,7 +1590,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="21518310"/>
+        <c:crossAx val="12868119"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1521,7 +1598,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="21518310"/>
+        <c:axId val="12868119"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1563,7 +1640,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="45375014"/>
+        <c:crossAx val="28970228"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1598,13 +1675,13 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>-354600</xdr:colOff>
       <xdr:row>42</xdr:row>
-      <xdr:rowOff>157680</xdr:rowOff>
+      <xdr:rowOff>7200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>57</xdr:row>
-      <xdr:rowOff>179640</xdr:rowOff>
+      <xdr:rowOff>29160</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1806,7 +1883,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:F30"/>
+  <dimension ref="B2:F31"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -1850,7 +1927,7 @@
       </c>
       <c r="F6" s="6" t="n">
         <f aca="false">'المقارنات السعرية'!E30</f>
-        <v>1300000</v>
+        <v>1327777.77777778</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1866,7 +1943,7 @@
       </c>
       <c r="F7" s="6" t="n">
         <f aca="false">'المقارنات السعرية'!F30</f>
-        <v>1500000</v>
+        <v>1550000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1882,7 +1959,7 @@
       </c>
       <c r="F8" s="8" t="str">
         <f aca="false">'المقارنات السعرية'!I34&amp;" من "&amp;'المقارنات السعرية'!D30</f>
-        <v>7 من 7</v>
+        <v>9 من 9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1890,7 +1967,7 @@
         <v>10</v>
       </c>
       <c r="C9" s="6" t="n">
-        <f aca="false">'المقارنات السعرية'!J13</f>
+        <f aca="false">'المقارنات السعرية'!J15</f>
         <v>4202.60195877796</v>
       </c>
       <c r="E9" s="4" t="s">
@@ -1898,7 +1975,7 @@
       </c>
       <c r="F9" s="9" t="n">
         <f aca="false">'المقارنات السعرية'!I36</f>
-        <v>0.115384615384615</v>
+        <v>0.133891213389121</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1914,7 +1991,7 @@
       </c>
       <c r="F10" s="10" t="n">
         <f aca="false">'المقارنات السعرية'!G30</f>
-        <v>235.142857142857</v>
+        <v>243.777777777778</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2020,7 +2097,7 @@
       </c>
       <c r="F18" s="9" t="n">
         <f aca="false">'العائد على المستثمر'!C47</f>
-        <v>0.0576923076923077</v>
+        <v>0.0564853556485356</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2035,7 +2112,7 @@
     <row r="21" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="12" t="str">
         <f aca="false">"• "&amp;F8&amp;" تاون هاوس في القادسية معروضة بأعلى من سعرنا، تصل إلى "&amp;TEXT(F7,"#,##0")&amp;" ريال – ومتوسط الحي "&amp;TEXT(F6,"#,##0")&amp;" ريال."</f>
-        <v>• 7 من 7 تاون هاوس في القادسية معروضة بأعلى من سعرنا، تصل إلى 1,500,000 ريال – ومتوسط الحي 1,300,000 ريال.</v>
+        <v>• 9 من 9 تاون هاوس في القادسية معروضة بأعلى من سعرنا، تصل إلى 1,550,000 ريال – ومتوسط الحي 1,327,778 ريال.</v>
       </c>
       <c r="C21" s="12"/>
       <c r="D21" s="12"/>
@@ -2045,7 +2122,7 @@
     <row r="22" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="12" t="str">
         <f aca="false">"• وحدتنا "&amp;TEXT(C8,"#,##0")&amp;" م² على 4 مستويات مقابل متوسط "&amp;TEXT(F10,"#,##0")&amp;" م² في الحي – مساحة أكبر بسعر أقل."</f>
-        <v>• وحدتنا 274 م² على 4 مستويات مقابل متوسط 235 م² في الحي – مساحة أكبر بسعر أقل.</v>
+        <v>• وحدتنا 274 م² على 4 مستويات مقابل متوسط 244 م² في الحي – مساحة أكبر بسعر أقل.</v>
       </c>
       <c r="C22" s="12"/>
       <c r="D22" s="12"/>
@@ -2062,8 +2139,9 @@
       <c r="F23" s="12"/>
     </row>
     <row r="24" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="12" t="s">
-        <v>30</v>
+      <c r="B24" s="12" t="str">
+        <f aca="false">"• الفلل المستقلة في القادسية معروضة من "&amp;TEXT(MIN('المقارنات السعرية'!I65:I69),"#,##0")&amp;" حتى "&amp;TEXT(MAX('المقارنات السعرية'!I65:I69),"#,##0")&amp;" ريال – ووحدتنا تقدم مواصفات قريبة منها (مصعد، قبو، ملحق) بسعر "&amp;TEXT(C7,"#,##0")&amp;"."</f>
+        <v>• الفلل المستقلة في القادسية معروضة من 1,600,000 حتى 2,150,000 ريال – ووحدتنا تقدم مواصفات قريبة منها (مصعد، قبو، ملحق) بسعر 1,150,000.</v>
       </c>
       <c r="C24" s="12"/>
       <c r="D24" s="12"/>
@@ -2072,7 +2150,7 @@
     </row>
     <row r="25" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C25" s="12"/>
       <c r="D25" s="12"/>
@@ -2081,7 +2159,7 @@
     </row>
     <row r="26" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C26" s="12"/>
       <c r="D26" s="12"/>
@@ -2089,33 +2167,42 @@
       <c r="F26" s="12"/>
     </row>
     <row r="27" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="12" t="str">
-        <f aca="false">"• للتأجير: عائد إجمالي "&amp;TEXT(F16,"0.0%")&amp;" على سعر الشراء مقابل "&amp;TEXT(F18,"0.0%")&amp;" لمن يشتري بمتوسط سعر الحي."</f>
-        <v>• للتأجير: عائد إجمالي 6.5% على سعر الشراء مقابل 5.8% لمن يشتري بمتوسط سعر الحي.</v>
+      <c r="B27" s="12" t="s">
+        <v>32</v>
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="12"/>
       <c r="E27" s="12"/>
       <c r="F27" s="12"/>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="13" t="s">
+    <row r="28" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B28" s="12" t="str">
+        <f aca="false">"• للتأجير: عائد إجمالي "&amp;TEXT(F16,"0.0%")&amp;" على سعر الشراء مقابل "&amp;TEXT(F18,"0.0%")&amp;" لمن يشتري بمتوسط سعر الحي."</f>
+        <v>• للتأجير: عائد إجمالي 6.5% على سعر الشراء مقابل 5.6% لمن يشتري بمتوسط سعر الحي.</v>
+      </c>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="12"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B30" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="13"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="13"/>
       <c r="C30" s="13"/>
       <c r="D30" s="13"/>
       <c r="E30" s="13"/>
       <c r="F30" s="13"/>
     </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="13"/>
+    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="B13:C13"/>
@@ -2128,7 +2215,8 @@
     <mergeCell ref="B25:F25"/>
     <mergeCell ref="B26:F26"/>
     <mergeCell ref="B27:F27"/>
-    <mergeCell ref="B29:F30"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B30:F31"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2216,7 +2304,7 @@
       </c>
       <c r="D8" s="4" t="str">
         <f aca="false">"متوسط "&amp;TEXT('المقارنات السعرية'!G30,"#,##0")&amp;" م²"</f>
-        <v>متوسط 235 م²</v>
+        <v>متوسط 244 م²</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>49</v>
@@ -2358,7 +2446,7 @@
       </c>
       <c r="D18" s="4" t="str">
         <f aca="false">TEXT('المقارنات السعرية'!E30,"#,##0")&amp;" متوسط – حتى "&amp;TEXT('المقارنات السعرية'!F30,"#,##0")</f>
-        <v>1,300,000 متوسط – حتى 1,500,000</v>
+        <v>1,327,778 متوسط – حتى 1,550,000</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>87</v>
@@ -2752,7 +2840,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:L44"/>
+  <dimension ref="B2:L72"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -2829,24 +2917,24 @@
       <c r="F6" s="31" t="s">
         <v>161</v>
       </c>
-      <c r="G6" s="32" t="s">
+      <c r="G6" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H6" s="32" t="n">
+        <v>360</v>
+      </c>
+      <c r="I6" s="33" t="n">
+        <v>1550000</v>
+      </c>
+      <c r="J6" s="34" t="n">
+        <f aca="false">IFERROR(I6/H6,0)</f>
+        <v>4305.55555555556</v>
+      </c>
+      <c r="K6" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="H6" s="33" t="n">
-        <v>300</v>
-      </c>
-      <c r="I6" s="34" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="J6" s="35" t="n">
-        <f aca="false">IFERROR(I6/H6,0)</f>
-        <v>5000</v>
-      </c>
-      <c r="K6" s="29" t="s">
+      <c r="L6" s="35" t="s">
         <v>163</v>
-      </c>
-      <c r="L6" s="36" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2857,32 +2945,32 @@
         <v>158</v>
       </c>
       <c r="D7" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="E7" s="29" t="s">
         <v>165</v>
       </c>
-      <c r="E7" s="29" t="s">
+      <c r="F7" s="36" t="s">
         <v>166</v>
       </c>
-      <c r="F7" s="37" t="s">
-        <v>59</v>
-      </c>
-      <c r="G7" s="32" t="s">
+      <c r="G7" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H7" s="32" t="n">
+        <v>300</v>
+      </c>
+      <c r="I7" s="33" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="J7" s="34" t="n">
+        <f aca="false">IFERROR(I7/H7,0)</f>
+        <v>5000</v>
+      </c>
+      <c r="K7" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="H7" s="33" t="n">
-        <v>250</v>
-      </c>
-      <c r="I7" s="34" t="n">
-        <v>1400000</v>
-      </c>
-      <c r="J7" s="35" t="n">
-        <f aca="false">IFERROR(I7/H7,0)</f>
-        <v>5600</v>
-      </c>
-      <c r="K7" s="29" t="s">
-        <v>163</v>
-      </c>
-      <c r="L7" s="36" t="s">
-        <v>164</v>
+      <c r="L7" s="35" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2893,32 +2981,32 @@
         <v>158</v>
       </c>
       <c r="D8" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="E8" s="29" t="s">
+        <v>169</v>
+      </c>
+      <c r="F8" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="G8" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H8" s="32" t="n">
+        <v>250</v>
+      </c>
+      <c r="I8" s="33" t="n">
+        <v>1400000</v>
+      </c>
+      <c r="J8" s="34" t="n">
+        <f aca="false">IFERROR(I8/H8,0)</f>
+        <v>5600</v>
+      </c>
+      <c r="K8" s="29" t="s">
+        <v>162</v>
+      </c>
+      <c r="L8" s="35" t="s">
         <v>167</v>
-      </c>
-      <c r="E8" s="29" t="s">
-        <v>168</v>
-      </c>
-      <c r="F8" s="31" t="s">
-        <v>169</v>
-      </c>
-      <c r="G8" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="H8" s="33" t="n">
-        <v>248</v>
-      </c>
-      <c r="I8" s="34" t="n">
-        <v>1350000</v>
-      </c>
-      <c r="J8" s="35" t="n">
-        <f aca="false">IFERROR(I8/H8,0)</f>
-        <v>5443.54838709678</v>
-      </c>
-      <c r="K8" s="29" t="s">
-        <v>163</v>
-      </c>
-      <c r="L8" s="36" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2929,35 +3017,35 @@
         <v>158</v>
       </c>
       <c r="D9" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="E9" s="29" t="s">
         <v>171</v>
       </c>
-      <c r="E9" s="29" t="s">
+      <c r="F9" s="36" t="s">
         <v>172</v>
       </c>
-      <c r="F9" s="32" t="s">
+      <c r="G9" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H9" s="32" t="n">
+        <v>248</v>
+      </c>
+      <c r="I9" s="33" t="n">
+        <v>1350000</v>
+      </c>
+      <c r="J9" s="34" t="n">
+        <f aca="false">IFERROR(I9/H9,0)</f>
+        <v>5443.54838709678</v>
+      </c>
+      <c r="K9" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="G9" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="H9" s="33" t="n">
-        <v>215</v>
-      </c>
-      <c r="I9" s="34" t="n">
-        <v>1250000</v>
-      </c>
-      <c r="J9" s="35" t="n">
-        <f aca="false">IFERROR(I9/H9,0)</f>
-        <v>5813.95348837209</v>
-      </c>
-      <c r="K9" s="29" t="s">
-        <v>163</v>
-      </c>
-      <c r="L9" s="36" t="s">
+      <c r="L9" s="35" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="29" t="n">
         <v>5</v>
       </c>
@@ -2968,29 +3056,29 @@
         <v>174</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>166</v>
-      </c>
-      <c r="F10" s="37" t="s">
-        <v>59</v>
-      </c>
-      <c r="G10" s="32" t="s">
+        <v>171</v>
+      </c>
+      <c r="F10" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="G10" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H10" s="32" t="n">
+        <v>188</v>
+      </c>
+      <c r="I10" s="33" t="n">
+        <v>1300000</v>
+      </c>
+      <c r="J10" s="34" t="n">
+        <f aca="false">IFERROR(I10/H10,0)</f>
+        <v>6914.89361702128</v>
+      </c>
+      <c r="K10" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="H10" s="33" t="n">
-        <v>225</v>
-      </c>
-      <c r="I10" s="34" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="J10" s="35" t="n">
-        <f aca="false">IFERROR(I10/H10,0)</f>
-        <v>5333.33333333333</v>
-      </c>
-      <c r="K10" s="29" t="s">
-        <v>175</v>
-      </c>
-      <c r="L10" s="36" t="s">
-        <v>176</v>
+      <c r="L10" s="35" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3001,32 +3089,32 @@
         <v>158</v>
       </c>
       <c r="D11" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="E11" s="29" t="s">
+        <v>176</v>
+      </c>
+      <c r="F11" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="G11" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H11" s="32" t="n">
+        <v>215</v>
+      </c>
+      <c r="I11" s="33" t="n">
+        <v>1250000</v>
+      </c>
+      <c r="J11" s="34" t="n">
+        <f aca="false">IFERROR(I11/H11,0)</f>
+        <v>5813.95348837209</v>
+      </c>
+      <c r="K11" s="29" t="s">
+        <v>162</v>
+      </c>
+      <c r="L11" s="35" t="s">
         <v>177</v>
-      </c>
-      <c r="E11" s="29" t="s">
-        <v>178</v>
-      </c>
-      <c r="F11" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="G11" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="H11" s="33" t="n">
-        <v>220</v>
-      </c>
-      <c r="I11" s="34" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="J11" s="35" t="n">
-        <f aca="false">IFERROR(I11/H11,0)</f>
-        <v>5454.54545454546</v>
-      </c>
-      <c r="K11" s="29" t="s">
-        <v>179</v>
-      </c>
-      <c r="L11" s="36" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3037,97 +3125,169 @@
         <v>158</v>
       </c>
       <c r="D12" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="E12" s="29" t="s">
+        <v>169</v>
+      </c>
+      <c r="F12" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="G12" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H12" s="32" t="n">
+        <v>225</v>
+      </c>
+      <c r="I12" s="33" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="J12" s="34" t="n">
+        <f aca="false">IFERROR(I12/H12,0)</f>
+        <v>5333.33333333333</v>
+      </c>
+      <c r="K12" s="29" t="s">
+        <v>179</v>
+      </c>
+      <c r="L12" s="35" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="29" t="n">
+        <v>8</v>
+      </c>
+      <c r="C13" s="30" t="s">
+        <v>158</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="E12" s="29" t="s">
-        <v>168</v>
-      </c>
-      <c r="F12" s="32" t="s">
+      <c r="E13" s="29" t="s">
+        <v>160</v>
+      </c>
+      <c r="F13" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="G13" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H13" s="32" t="n">
+        <v>220</v>
+      </c>
+      <c r="I13" s="33" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="J13" s="34" t="n">
+        <f aca="false">IFERROR(I13/H13,0)</f>
+        <v>5454.54545454546</v>
+      </c>
+      <c r="K13" s="29" t="s">
+        <v>182</v>
+      </c>
+      <c r="L13" s="35" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="29" t="n">
+        <v>9</v>
+      </c>
+      <c r="C14" s="30" t="s">
+        <v>158</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E14" s="29" t="s">
+        <v>171</v>
+      </c>
+      <c r="F14" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="G14" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H14" s="32" t="n">
+        <v>188</v>
+      </c>
+      <c r="I14" s="33" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="J14" s="34" t="n">
+        <f aca="false">IFERROR(I14/H14,0)</f>
+        <v>6382.97872340426</v>
+      </c>
+      <c r="K14" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="G12" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="H12" s="33" t="n">
+      <c r="L14" s="35" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="38" t="s">
+        <v>186</v>
+      </c>
+      <c r="C15" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="D15" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="E15" s="38" t="s">
         <v>188</v>
       </c>
-      <c r="I12" s="34" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="J12" s="35" t="n">
-        <f aca="false">IFERROR(I12/H12,0)</f>
-        <v>6382.97872340426</v>
-      </c>
-      <c r="K12" s="29" t="s">
-        <v>163</v>
-      </c>
-      <c r="L12" s="36" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="38" t="s">
-        <v>183</v>
-      </c>
-      <c r="C13" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="D13" s="16" t="s">
-        <v>184</v>
-      </c>
-      <c r="E13" s="38" t="s">
-        <v>185</v>
-      </c>
-      <c r="F13" s="38" t="s">
-        <v>186</v>
-      </c>
-      <c r="G13" s="38" t="s">
-        <v>187</v>
-      </c>
-      <c r="H13" s="39" t="n">
+      <c r="F15" s="38" t="s">
+        <v>189</v>
+      </c>
+      <c r="G15" s="38" t="s">
+        <v>190</v>
+      </c>
+      <c r="H15" s="39" t="n">
         <f aca="false">الافتراضات!$C$13</f>
         <v>273.64</v>
       </c>
-      <c r="I13" s="11" t="n">
+      <c r="I15" s="11" t="n">
         <f aca="false">الافتراضات!$C$8</f>
         <v>1150000</v>
       </c>
-      <c r="J13" s="40" t="n">
-        <f aca="false">IFERROR(I13/H13,0)</f>
+      <c r="J15" s="40" t="n">
+        <f aca="false">IFERROR(I15/H15,0)</f>
         <v>4202.60195877796</v>
       </c>
-      <c r="K13" s="38" t="s">
-        <v>188</v>
-      </c>
-      <c r="L13" s="16" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D14" s="41" t="s">
-        <v>190</v>
-      </c>
-      <c r="H14" s="39" t="n">
+      <c r="K15" s="38" t="s">
+        <v>191</v>
+      </c>
+      <c r="L15" s="16" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D16" s="41" t="s">
+        <v>193</v>
+      </c>
+      <c r="H16" s="39" t="n">
         <f aca="false">الافتراضات!$C$14</f>
         <v>202.24</v>
       </c>
-      <c r="I14" s="11" t="n">
+      <c r="I16" s="11" t="n">
         <f aca="false">الافتراضات!$C$8</f>
         <v>1150000</v>
       </c>
-      <c r="J14" s="40" t="n">
-        <f aca="false">IFERROR(I14/H14,0)</f>
+      <c r="J16" s="40" t="n">
+        <f aca="false">IFERROR(I16/H16,0)</f>
         <v>5686.31329113924</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D15" s="2" t="s">
-        <v>191</v>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D17" s="2" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="3" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
@@ -3145,19 +3305,19 @@
         <v>149</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="G29" s="14" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="H29" s="14" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3165,54 +3325,54 @@
         <v>158</v>
       </c>
       <c r="D30" s="42" t="n">
-        <f aca="false">COUNTIF($C$6:$C$12,C30)</f>
-        <v>7</v>
-      </c>
-      <c r="E30" s="35" t="n">
-        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$12,C30,$I$6:$I$12),0)</f>
-        <v>1300000</v>
-      </c>
-      <c r="F30" s="35" t="n">
-        <f aca="false">_xlfn.MAXIFS($I$6:$I$12,$C$6:$C$12,C30)</f>
-        <v>1500000</v>
+        <f aca="false">COUNTIF($C$6:$C$14,C30)</f>
+        <v>9</v>
+      </c>
+      <c r="E30" s="34" t="n">
+        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$14,C30,$I$6:$I$14),0)</f>
+        <v>1327777.77777778</v>
+      </c>
+      <c r="F30" s="34" t="n">
+        <f aca="false">_xlfn.MAXIFS($I$6:$I$14,$C$6:$C$14,C30)</f>
+        <v>1550000</v>
       </c>
       <c r="G30" s="43" t="n">
-        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$12,C30,$H$6:$H$12),0)</f>
-        <v>235.142857142857</v>
+        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$14,C30,$H$6:$H$14),0)</f>
+        <v>243.777777777778</v>
       </c>
       <c r="H30" s="28" t="n">
-        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$12,C30,$J$6:$J$12),0)</f>
-        <v>5575.47991239313</v>
+        <f aca="false">IFERROR(AVERAGEIF($C$6:$C$14,C30,$J$6:$J$14),0)</f>
+        <v>5583.20095103653</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C31" s="38" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="D31" s="44" t="n">
         <f aca="false">الافتراضات!$C$7</f>
         <v>12</v>
       </c>
       <c r="E31" s="40" t="n">
-        <f aca="false">I13</f>
+        <f aca="false">I15</f>
         <v>1150000</v>
       </c>
       <c r="F31" s="40" t="n">
-        <f aca="false">I13</f>
+        <f aca="false">I15</f>
         <v>1150000</v>
       </c>
       <c r="G31" s="45" t="n">
-        <f aca="false">H13</f>
+        <f aca="false">H15</f>
         <v>273.64</v>
       </c>
       <c r="H31" s="40" t="n">
-        <f aca="false">J13</f>
+        <f aca="false">J15</f>
         <v>4202.60195877796</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="3" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
@@ -3227,7 +3387,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C34" s="15" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D34" s="15"/>
       <c r="E34" s="15"/>
@@ -3235,13 +3395,13 @@
       <c r="G34" s="15"/>
       <c r="H34" s="15"/>
       <c r="I34" s="46" t="n">
-        <f aca="false">COUNTIFS($C$6:$C$12,"القادسية",$I$6:$I$12,"&gt;"&amp;I13)</f>
-        <v>7</v>
+        <f aca="false">COUNTIFS($C$6:$C$14,"القادسية",$I$6:$I$14,"&gt;"&amp;I15)</f>
+        <v>9</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C35" s="15" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="D35" s="15"/>
       <c r="E35" s="15"/>
@@ -3250,12 +3410,12 @@
       <c r="H35" s="15"/>
       <c r="I35" s="40" t="n">
         <f aca="false">E30-E31</f>
-        <v>150000</v>
+        <v>177777.777777778</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C36" s="15" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="D36" s="15"/>
       <c r="E36" s="15"/>
@@ -3264,12 +3424,12 @@
       <c r="H36" s="15"/>
       <c r="I36" s="47" t="n">
         <f aca="false">IFERROR(1-E31/E30,0)</f>
-        <v>0.115384615384615</v>
+        <v>0.133891213389121</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C37" s="15" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D37" s="15"/>
       <c r="E37" s="15"/>
@@ -3278,12 +3438,12 @@
       <c r="H37" s="15"/>
       <c r="I37" s="47" t="n">
         <f aca="false">IFERROR(1-E31/F30,0)</f>
-        <v>0.233333333333333</v>
+        <v>0.258064516129032</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C38" s="15" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D38" s="15"/>
       <c r="E38" s="15"/>
@@ -3292,12 +3452,12 @@
       <c r="H38" s="15"/>
       <c r="I38" s="45" t="n">
         <f aca="false">G31-G30</f>
-        <v>38.4971428571429</v>
+        <v>29.8622222222222</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C39" s="15" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="D39" s="15"/>
       <c r="E39" s="15"/>
@@ -3306,12 +3466,12 @@
       <c r="H39" s="15"/>
       <c r="I39" s="47" t="n">
         <f aca="false">IFERROR(1-H31/H30,0)</f>
-        <v>0.246234938550052</v>
+        <v>0.247277324310217</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C40" s="15" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="D40" s="15"/>
       <c r="E40" s="15"/>
@@ -3319,13 +3479,13 @@
       <c r="G40" s="15"/>
       <c r="H40" s="15"/>
       <c r="I40" s="47" t="n">
-        <f aca="false">IFERROR(1-J14/H30,0)</f>
-        <v>-0.019878715462637</v>
+        <f aca="false">IFERROR(1-J16/H30,0)</f>
+        <v>-0.0184683196981421</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C42" s="13" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D42" s="13"/>
       <c r="E42" s="13"/>
@@ -3361,8 +3521,257 @@
       <c r="K44" s="13"/>
       <c r="L44" s="13"/>
     </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B63" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="C63" s="3"/>
+      <c r="D63" s="3"/>
+      <c r="E63" s="3"/>
+      <c r="F63" s="3"/>
+      <c r="G63" s="3"/>
+      <c r="H63" s="3"/>
+      <c r="I63" s="3"/>
+      <c r="J63" s="3"/>
+      <c r="K63" s="3"/>
+      <c r="L63" s="3"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B64" s="14" t="s">
+        <v>148</v>
+      </c>
+      <c r="C64" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="D64" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="E64" s="14" t="s">
+        <v>212</v>
+      </c>
+      <c r="F64" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="G64" s="14"/>
+      <c r="H64" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="I64" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="J64" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="K64" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="L64" s="14" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B65" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" s="29" t="s">
+        <v>158</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="E65" s="29" t="s">
+        <v>214</v>
+      </c>
+      <c r="F65" s="37" t="s">
+        <v>215</v>
+      </c>
+      <c r="G65" s="29"/>
+      <c r="H65" s="32" t="n">
+        <v>275</v>
+      </c>
+      <c r="I65" s="33" t="n">
+        <v>2150000</v>
+      </c>
+      <c r="J65" s="34" t="n">
+        <f aca="false">IFERROR(I65/H65,0)</f>
+        <v>7818.18181818182</v>
+      </c>
+      <c r="K65" s="29" t="s">
+        <v>162</v>
+      </c>
+      <c r="L65" s="35" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B66" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="C66" s="29" t="s">
+        <v>158</v>
+      </c>
+      <c r="D66" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="E66" s="29" t="s">
+        <v>214</v>
+      </c>
+      <c r="F66" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="G66" s="29"/>
+      <c r="H66" s="32" t="n">
+        <v>247</v>
+      </c>
+      <c r="I66" s="33" t="n">
+        <v>1850000</v>
+      </c>
+      <c r="J66" s="34" t="n">
+        <f aca="false">IFERROR(I66/H66,0)</f>
+        <v>7489.87854251012</v>
+      </c>
+      <c r="K66" s="29" t="s">
+        <v>162</v>
+      </c>
+      <c r="L66" s="35" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B67" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="C67" s="29" t="s">
+        <v>158</v>
+      </c>
+      <c r="D67" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="E67" s="29" t="s">
+        <v>214</v>
+      </c>
+      <c r="F67" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="G67" s="29"/>
+      <c r="H67" s="32" t="n">
+        <v>333</v>
+      </c>
+      <c r="I67" s="33" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="J67" s="34" t="n">
+        <f aca="false">IFERROR(I67/H67,0)</f>
+        <v>5405.40540540541</v>
+      </c>
+      <c r="K67" s="29" t="s">
+        <v>162</v>
+      </c>
+      <c r="L67" s="35" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B68" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C68" s="29" t="s">
+        <v>158</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="E68" s="29" t="s">
+        <v>214</v>
+      </c>
+      <c r="F68" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="G68" s="29"/>
+      <c r="H68" s="32" t="n">
+        <v>285</v>
+      </c>
+      <c r="I68" s="33" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="J68" s="34" t="n">
+        <f aca="false">IFERROR(I68/H68,0)</f>
+        <v>6315.78947368421</v>
+      </c>
+      <c r="K68" s="29" t="s">
+        <v>162</v>
+      </c>
+      <c r="L68" s="35" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B69" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="C69" s="29" t="s">
+        <v>158</v>
+      </c>
+      <c r="D69" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="E69" s="29" t="s">
+        <v>214</v>
+      </c>
+      <c r="F69" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="G69" s="29"/>
+      <c r="H69" s="32" t="n">
+        <v>200</v>
+      </c>
+      <c r="I69" s="33" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="J69" s="34" t="n">
+        <f aca="false">IFERROR(I69/H69,0)</f>
+        <v>8000</v>
+      </c>
+      <c r="K69" s="29" t="s">
+        <v>162</v>
+      </c>
+      <c r="L69" s="35" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D70" s="48" t="s">
+        <v>224</v>
+      </c>
+      <c r="H70" s="49" t="n">
+        <f aca="false">AVERAGE(H65:H69)</f>
+        <v>268</v>
+      </c>
+      <c r="I70" s="50" t="n">
+        <f aca="false">AVERAGE(I65:I69)</f>
+        <v>1840000</v>
+      </c>
+      <c r="J70" s="50" t="n">
+        <f aca="false">AVERAGE(J65:J69)</f>
+        <v>7005.85104795631</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D71" s="16" t="s">
+        <v>225</v>
+      </c>
+      <c r="I71" s="47" t="n">
+        <f aca="false">IFERROR(1-I15/I70,0)</f>
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D72" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="B28:L28"/>
     <mergeCell ref="B33:L33"/>
     <mergeCell ref="C34:H34"/>
@@ -3373,20 +3782,28 @@
     <mergeCell ref="C39:H39"/>
     <mergeCell ref="C40:H40"/>
     <mergeCell ref="C42:L44"/>
+    <mergeCell ref="B63:L63"/>
   </mergeCells>
-  <conditionalFormatting sqref="I6:I12">
+  <conditionalFormatting sqref="I6:I14">
     <cfRule type="cellIs" priority="2" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>$I$13</formula>
+      <formula>$I$15</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="L6" r:id="rId1" display="https://haraj.com.sa/11140216303/"/>
+    <hyperlink ref="L6" r:id="rId1" display="https://haraj.com.sa/11151459820/"/>
     <hyperlink ref="L7" r:id="rId2" display="https://haraj.com.sa/11140216303/"/>
-    <hyperlink ref="L8" r:id="rId3" display="https://sa.aqar.fm/فلل-للبيع/الرياض/شرق-الرياض/حي-القادسية/تاون-هاوس"/>
-    <hyperlink ref="L9" r:id="rId4" display="https://www.bayut.sa/en/for-sale/villas/riyadh/east-riyadh/al-qadisiyah/"/>
-    <hyperlink ref="L10" r:id="rId5" display="https://haraj.com.sa/en/11164555558/"/>
-    <hyperlink ref="L11" r:id="rId6" display="https://haraj.com.sa/11151387860/"/>
-    <hyperlink ref="L12" r:id="rId7" display="https://www.bayut.sa/en/property/details-87578604.html"/>
+    <hyperlink ref="L8" r:id="rId3" display="https://haraj.com.sa/11140216303/"/>
+    <hyperlink ref="L9" r:id="rId4" display="https://sa.aqar.fm/فلل-للبيع/الرياض/شرق-الرياض/حي-القادسية/تاون-هاوس"/>
+    <hyperlink ref="L10" r:id="rId5" display="https://sa.aqar.fm/فلل-للبيع/الرياض/شرق-الرياض/حي-القادسية/تاون-هاوس"/>
+    <hyperlink ref="L11" r:id="rId6" display="https://www.bayut.sa/en/for-sale/villas/riyadh/east-riyadh/al-qadisiyah/"/>
+    <hyperlink ref="L12" r:id="rId7" display="https://haraj.com.sa/en/11164555558/"/>
+    <hyperlink ref="L13" r:id="rId8" display="https://haraj.com.sa/11151387860/"/>
+    <hyperlink ref="L14" r:id="rId9" display="https://www.bayut.sa/en/property/details-87578604.html"/>
+    <hyperlink ref="L65" r:id="rId10" display="https://www.bayut.sa/en/property/details-87614706.html"/>
+    <hyperlink ref="L66" r:id="rId11" display="https://sa.aqar.fm/فلل-للبيع/الرياض/شرق-الرياض/حي-القادسية"/>
+    <hyperlink ref="L67" r:id="rId12" display="https://haraj.com.sa/search/فيلا للبيع في حي القادسية في الرياض/"/>
+    <hyperlink ref="L68" r:id="rId13" display="https://www.propertyfinder.sa/en/buy/ar-riyadh/villas-for-sale-al-qadisiyah.html"/>
+    <hyperlink ref="L69" r:id="rId14" display="https://www.propertyfinder.sa/en/buy/ar-riyadh/villas-for-sale-al-qadisiyah.html"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3395,7 +3812,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId8"/>
+  <drawing r:id="rId15"/>
 </worksheet>
 </file>
 
@@ -3415,12 +3832,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="21.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>208</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>209</v>
+        <v>228</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -3431,25 +3848,25 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="C5" s="35" t="n">
+        <v>229</v>
+      </c>
+      <c r="C5" s="34" t="n">
         <f aca="false">الافتراضات!$C$7*الافتراضات!$C$8</f>
         <v>13800000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="C6" s="35" t="n">
+        <v>230</v>
+      </c>
+      <c r="C6" s="34" t="n">
         <f aca="false">C5*(الافتراضات!$C$16+الافتراضات!$C$17)</f>
         <v>690000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="15" t="s">
-        <v>212</v>
+        <v>231</v>
       </c>
       <c r="C7" s="28" t="n">
         <f aca="false">C5+C6</f>
@@ -3458,25 +3875,25 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="C8" s="35" t="n">
+        <v>232</v>
+      </c>
+      <c r="C8" s="34" t="n">
         <f aca="false">الافتراضات!$C$7*الافتراضات!$C$25</f>
         <v>16200000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="C9" s="35" t="n">
+        <v>233</v>
+      </c>
+      <c r="C9" s="34" t="n">
         <f aca="false">الافتراضات!$C$7*'المقارنات السعرية'!E30</f>
-        <v>15600000</v>
+        <v>15933333.3333333</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="15" t="s">
-        <v>215</v>
+        <v>234</v>
       </c>
       <c r="C10" s="40" t="n">
         <f aca="false">C8-C5</f>
@@ -3485,7 +3902,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
-        <v>216</v>
+        <v>235</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
@@ -3499,45 +3916,45 @@
         <v>91</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>217</v>
+        <v>236</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>218</v>
+        <v>237</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>219</v>
+        <v>238</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>220</v>
+        <v>239</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>221</v>
+        <v>240</v>
       </c>
       <c r="H13" s="14" t="s">
-        <v>222</v>
+        <v>241</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="C14" s="35" t="n">
+        <v>242</v>
+      </c>
+      <c r="C14" s="34" t="n">
         <f aca="false">-الافتراضات!$C$19*$C$5</f>
         <v>-13800000</v>
       </c>
-      <c r="D14" s="35" t="n">
+      <c r="D14" s="34" t="n">
         <f aca="false">-الافتراضات!$C$20*$C$5</f>
         <v>-0</v>
       </c>
-      <c r="E14" s="35" t="n">
+      <c r="E14" s="34" t="n">
         <f aca="false">-الافتراضات!$C$21*$C$5</f>
         <v>-0</v>
       </c>
-      <c r="F14" s="35" t="n">
+      <c r="F14" s="34" t="n">
         <f aca="false">-الافتراضات!$C$22*$C$5</f>
         <v>-0</v>
       </c>
-      <c r="G14" s="35" t="n">
+      <c r="G14" s="34" t="n">
         <f aca="false">-الافتراضات!$C$23*$C$5</f>
         <v>-0</v>
       </c>
@@ -3548,25 +3965,25 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="C15" s="35" t="n">
+        <v>243</v>
+      </c>
+      <c r="C15" s="34" t="n">
         <f aca="false">IF(0=0,-$C$6,0)</f>
         <v>-690000</v>
       </c>
-      <c r="D15" s="35" t="n">
+      <c r="D15" s="34" t="n">
         <f aca="false">IF(1=0,-$C$6,0)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="35" t="n">
+      <c r="E15" s="34" t="n">
         <f aca="false">IF(2=0,-$C$6,0)</f>
         <v>0</v>
       </c>
-      <c r="F15" s="35" t="n">
+      <c r="F15" s="34" t="n">
         <f aca="false">IF(3=0,-$C$6,0)</f>
         <v>0</v>
       </c>
-      <c r="G15" s="35" t="n">
+      <c r="G15" s="34" t="n">
         <f aca="false">IF(4=0,-$C$6,0)</f>
         <v>0</v>
       </c>
@@ -3577,25 +3994,25 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="C16" s="35" t="n">
+        <v>244</v>
+      </c>
+      <c r="C16" s="34" t="n">
         <f aca="false">IF(0*0.5=ROUND(الافتراضات!$C$28,1),الافتراضات!$C$7*الافتراضات!$C$29,0)</f>
         <v>0</v>
       </c>
-      <c r="D16" s="35" t="n">
+      <c r="D16" s="34" t="n">
         <f aca="false">IF(1*0.5=ROUND(الافتراضات!$C$28,1),الافتراضات!$C$7*الافتراضات!$C$29,0)</f>
         <v>0</v>
       </c>
-      <c r="E16" s="35" t="n">
+      <c r="E16" s="34" t="n">
         <f aca="false">IF(2*0.5=ROUND(الافتراضات!$C$28,1),الافتراضات!$C$7*الافتراضات!$C$29,0)</f>
         <v>0</v>
       </c>
-      <c r="F16" s="35" t="n">
+      <c r="F16" s="34" t="n">
         <f aca="false">IF(3*0.5=ROUND(الافتراضات!$C$28,1),الافتراضات!$C$7*الافتراضات!$C$29,0)</f>
         <v>0</v>
       </c>
-      <c r="G16" s="35" t="n">
+      <c r="G16" s="34" t="n">
         <f aca="false">IF(4*0.5=ROUND(الافتراضات!$C$28,1),الافتراضات!$C$7*الافتراضات!$C$29,0)</f>
         <v>16200000</v>
       </c>
@@ -3606,25 +4023,25 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="C17" s="35" t="n">
+        <v>245</v>
+      </c>
+      <c r="C17" s="34" t="n">
         <f aca="false">-C16*(الافتراضات!$C$30+الافتراضات!$C$31)</f>
         <v>-0</v>
       </c>
-      <c r="D17" s="35" t="n">
+      <c r="D17" s="34" t="n">
         <f aca="false">-D16*(الافتراضات!$C$30+الافتراضات!$C$31)</f>
         <v>-0</v>
       </c>
-      <c r="E17" s="35" t="n">
+      <c r="E17" s="34" t="n">
         <f aca="false">-E16*(الافتراضات!$C$30+الافتراضات!$C$31)</f>
         <v>-0</v>
       </c>
-      <c r="F17" s="35" t="n">
+      <c r="F17" s="34" t="n">
         <f aca="false">-F16*(الافتراضات!$C$30+الافتراضات!$C$31)</f>
         <v>-0</v>
       </c>
-      <c r="G17" s="35" t="n">
+      <c r="G17" s="34" t="n">
         <f aca="false">-G16*(الافتراضات!$C$30+الافتراضات!$C$31)</f>
         <v>-1215000</v>
       </c>
@@ -3635,54 +4052,54 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="15" t="s">
-        <v>227</v>
-      </c>
-      <c r="C18" s="48" t="n">
+        <v>246</v>
+      </c>
+      <c r="C18" s="50" t="n">
         <f aca="false">SUM(C14:C17)</f>
         <v>-14490000</v>
       </c>
-      <c r="D18" s="48" t="n">
+      <c r="D18" s="50" t="n">
         <f aca="false">SUM(D14:D17)</f>
         <v>0</v>
       </c>
-      <c r="E18" s="48" t="n">
+      <c r="E18" s="50" t="n">
         <f aca="false">SUM(E14:E17)</f>
         <v>0</v>
       </c>
-      <c r="F18" s="48" t="n">
+      <c r="F18" s="50" t="n">
         <f aca="false">SUM(F14:F17)</f>
         <v>0</v>
       </c>
-      <c r="G18" s="48" t="n">
+      <c r="G18" s="50" t="n">
         <f aca="false">SUM(G14:G17)</f>
         <v>14985000</v>
       </c>
-      <c r="H18" s="48" t="n">
+      <c r="H18" s="50" t="n">
         <f aca="false">SUM(C18:G18)</f>
         <v>495000</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="C19" s="35" t="n">
+        <v>247</v>
+      </c>
+      <c r="C19" s="34" t="n">
         <f aca="false">SUM($C$18:C18)</f>
         <v>-14490000</v>
       </c>
-      <c r="D19" s="35" t="n">
+      <c r="D19" s="34" t="n">
         <f aca="false">SUM($C$18:D18)</f>
         <v>-14490000</v>
       </c>
-      <c r="E19" s="35" t="n">
+      <c r="E19" s="34" t="n">
         <f aca="false">SUM($C$18:E18)</f>
         <v>-14490000</v>
       </c>
-      <c r="F19" s="35" t="n">
+      <c r="F19" s="34" t="n">
         <f aca="false">SUM($C$18:F18)</f>
         <v>-14490000</v>
       </c>
-      <c r="G19" s="35" t="n">
+      <c r="G19" s="34" t="n">
         <f aca="false">SUM($C$18:G18)</f>
         <v>495000</v>
       </c>
@@ -3693,7 +4110,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
-        <v>229</v>
+        <v>248</v>
       </c>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
@@ -3704,7 +4121,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="15" t="s">
-        <v>230</v>
+        <v>249</v>
       </c>
       <c r="C22" s="40" t="n">
         <f aca="false">H18</f>
@@ -3713,7 +4130,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="15" t="s">
-        <v>231</v>
+        <v>250</v>
       </c>
       <c r="C23" s="47" t="n">
         <f aca="false">IFERROR(H18/-SUMIF(C18:G18,"&lt;0"),0)</f>
@@ -3722,7 +4139,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="15" t="s">
-        <v>232</v>
+        <v>251</v>
       </c>
       <c r="C24" s="47" t="n">
         <f aca="false">IFERROR(C23/الافتراضات!$C$28,0)</f>
@@ -3731,7 +4148,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="15" t="s">
-        <v>233</v>
+        <v>252</v>
       </c>
       <c r="C25" s="47" t="n">
         <f aca="false">IFERROR((1+IRR(C18:G18))^2-1,0)</f>
@@ -3740,7 +4157,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="15" t="s">
-        <v>234</v>
+        <v>253</v>
       </c>
       <c r="C26" s="40" t="n">
         <f aca="false">IFERROR(C7/(1-الافتراضات!$C$30-الافتراضات!$C$31)/الافتراضات!$C$7,0)</f>
@@ -3749,7 +4166,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="15" t="s">
-        <v>235</v>
+        <v>254</v>
       </c>
       <c r="C27" s="47" t="n">
         <f aca="false">IFERROR(1-C26/الافتراضات!$C$29,0)</f>
@@ -3758,7 +4175,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="3" t="s">
-        <v>236</v>
+        <v>255</v>
       </c>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
@@ -3769,33 +4186,33 @@
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="14" t="s">
-        <v>237</v>
+        <v>256</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>238</v>
+        <v>257</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>239</v>
+        <v>258</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>240</v>
+        <v>259</v>
       </c>
       <c r="F30" s="14" t="s">
-        <v>239</v>
+        <v>258</v>
       </c>
       <c r="G30" s="14" t="s">
-        <v>241</v>
+        <v>260</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="49" t="n">
+      <c r="B31" s="51" t="n">
         <v>1200000</v>
       </c>
       <c r="C31" s="28" t="n">
         <f aca="false">الافتراضات!$C$7*B31*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)</f>
         <v>-1170000</v>
       </c>
-      <c r="D31" s="50" t="n">
+      <c r="D31" s="52" t="n">
         <f aca="false">IFERROR(C31/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)),0)</f>
         <v>-0.080745341614907</v>
       </c>
@@ -3803,24 +4220,24 @@
         <f aca="false">الافتراضات!$C$7*B31*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)</f>
         <v>-480000.000000002</v>
       </c>
-      <c r="F31" s="50" t="n">
+      <c r="F31" s="52" t="n">
         <f aca="false">IFERROR(E31/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)),0)</f>
         <v>-0.0347826086956523</v>
       </c>
-      <c r="G31" s="50" t="n">
+      <c r="G31" s="52" t="n">
         <f aca="false">IFERROR((الافتراضات!$C$7*B31*(1-الافتراضات!$C$30-الافتراضات!$C$31)/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)))^(1/الافتراضات!$C$28)-1,0)</f>
         <v>-0.0175452217509715</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="49" t="n">
+      <c r="B32" s="51" t="n">
         <v>1250000</v>
       </c>
       <c r="C32" s="28" t="n">
         <f aca="false">الافتراضات!$C$7*B32*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)</f>
         <v>-615000.000000002</v>
       </c>
-      <c r="D32" s="50" t="n">
+      <c r="D32" s="52" t="n">
         <f aca="false">IFERROR(C32/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)),0)</f>
         <v>-0.0424430641821948</v>
       </c>
@@ -3828,24 +4245,24 @@
         <f aca="false">الافتراضات!$C$7*B32*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)</f>
         <v>74999.9999999981</v>
       </c>
-      <c r="F32" s="50" t="n">
+      <c r="F32" s="52" t="n">
         <f aca="false">IFERROR(E32/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)),0)</f>
         <v>0.00543478260869552</v>
       </c>
-      <c r="G32" s="50" t="n">
+      <c r="G32" s="52" t="n">
         <f aca="false">IFERROR((الافتراضات!$C$7*B32*(1-الافتراضات!$C$30-الافتراضات!$C$31)/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)))^(1/الافتراضات!$C$28)-1,0)</f>
         <v>0.0027137091955487</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="49" t="n">
+      <c r="B33" s="51" t="n">
         <v>1300000</v>
       </c>
       <c r="C33" s="28" t="n">
         <f aca="false">الافتراضات!$C$7*B33*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)</f>
         <v>-60000.0000000019</v>
       </c>
-      <c r="D33" s="50" t="n">
+      <c r="D33" s="52" t="n">
         <f aca="false">IFERROR(C33/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)),0)</f>
         <v>-0.00414078674948253</v>
       </c>
@@ -3853,24 +4270,24 @@
         <f aca="false">الافتراضات!$C$7*B33*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)</f>
         <v>629999.999999998</v>
       </c>
-      <c r="F33" s="50" t="n">
+      <c r="F33" s="52" t="n">
         <f aca="false">IFERROR(E33/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)),0)</f>
         <v>0.0456521739130434</v>
       </c>
-      <c r="G33" s="50" t="n">
+      <c r="G33" s="52" t="n">
         <f aca="false">IFERROR((الافتراضات!$C$7*B33*(1-الافتراضات!$C$30-الافتراضات!$C$31)/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)))^(1/الافتراضات!$C$28)-1,0)</f>
         <v>0.0225713539470209</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="49" t="n">
+      <c r="B34" s="51" t="n">
         <v>1350000</v>
       </c>
       <c r="C34" s="28" t="n">
         <f aca="false">الافتراضات!$C$7*B34*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)</f>
         <v>494999.999999998</v>
       </c>
-      <c r="D34" s="50" t="n">
+      <c r="D34" s="52" t="n">
         <f aca="false">IFERROR(C34/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)),0)</f>
         <v>0.0341614906832297</v>
       </c>
@@ -3878,24 +4295,24 @@
         <f aca="false">الافتراضات!$C$7*B34*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)</f>
         <v>1185000</v>
       </c>
-      <c r="F34" s="50" t="n">
+      <c r="F34" s="52" t="n">
         <f aca="false">IFERROR(E34/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)),0)</f>
         <v>0.0858695652173912</v>
       </c>
-      <c r="G34" s="50" t="n">
+      <c r="G34" s="52" t="n">
         <f aca="false">IFERROR((الافتراضات!$C$7*B34*(1-الافتراضات!$C$30-الافتراضات!$C$31)/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)))^(1/الافتراضات!$C$28)-1,0)</f>
         <v>0.0420506538635208</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="49" t="n">
+      <c r="B35" s="51" t="n">
         <v>1400000</v>
       </c>
       <c r="C35" s="28" t="n">
         <f aca="false">الافتراضات!$C$7*B35*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)</f>
         <v>1050000</v>
       </c>
-      <c r="D35" s="50" t="n">
+      <c r="D35" s="52" t="n">
         <f aca="false">IFERROR(C35/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)),0)</f>
         <v>0.0724637681159419</v>
       </c>
@@ -3903,24 +4320,24 @@
         <f aca="false">الافتراضات!$C$7*B35*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)</f>
         <v>1740000</v>
       </c>
-      <c r="F35" s="50" t="n">
+      <c r="F35" s="52" t="n">
         <f aca="false">IFERROR(E35/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)),0)</f>
         <v>0.126086956521739</v>
       </c>
-      <c r="G35" s="50" t="n">
+      <c r="G35" s="52" t="n">
         <f aca="false">IFERROR((الافتراضات!$C$7*B35*(1-الافتراضات!$C$30-الافتراضات!$C$31)/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)))^(1/الافتراضات!$C$28)-1,0)</f>
         <v>0.0611724442906247</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="49" t="n">
+      <c r="B36" s="51" t="n">
         <v>1450000</v>
       </c>
       <c r="C36" s="28" t="n">
         <f aca="false">الافتراضات!$C$7*B36*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)</f>
         <v>1605000</v>
       </c>
-      <c r="D36" s="50" t="n">
+      <c r="D36" s="52" t="n">
         <f aca="false">IFERROR(C36/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)),0)</f>
         <v>0.110766045548654</v>
       </c>
@@ -3928,24 +4345,24 @@
         <f aca="false">الافتراضات!$C$7*B36*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)</f>
         <v>2295000</v>
       </c>
-      <c r="F36" s="50" t="n">
+      <c r="F36" s="52" t="n">
         <f aca="false">IFERROR(E36/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)),0)</f>
         <v>0.166304347826087</v>
       </c>
-      <c r="G36" s="50" t="n">
+      <c r="G36" s="52" t="n">
         <f aca="false">IFERROR((الافتراضات!$C$7*B36*(1-الافتراضات!$C$30-الافتراضات!$C$31)/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)))^(1/الافتراضات!$C$28)-1,0)</f>
         <v>0.079955715678234</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="49" t="n">
+      <c r="B37" s="51" t="n">
         <v>1500000</v>
       </c>
       <c r="C37" s="28" t="n">
         <f aca="false">الافتراضات!$C$7*B37*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)</f>
         <v>2160000</v>
       </c>
-      <c r="D37" s="50" t="n">
+      <c r="D37" s="52" t="n">
         <f aca="false">IFERROR(C37/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)),0)</f>
         <v>0.149068322981366</v>
       </c>
@@ -3953,24 +4370,24 @@
         <f aca="false">الافتراضات!$C$7*B37*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)</f>
         <v>2850000</v>
       </c>
-      <c r="F37" s="50" t="n">
+      <c r="F37" s="52" t="n">
         <f aca="false">IFERROR(E37/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)),0)</f>
         <v>0.206521739130435</v>
       </c>
-      <c r="G37" s="50" t="n">
+      <c r="G37" s="52" t="n">
         <f aca="false">IFERROR((الافتراضات!$C$7*B37*(1-الافتراضات!$C$30-الافتراضات!$C$31)/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)))^(1/الافتراضات!$C$28)-1,0)</f>
         <v>0.0984178344921547</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="49" t="n">
+      <c r="B38" s="51" t="n">
         <v>1550000</v>
       </c>
       <c r="C38" s="28" t="n">
         <f aca="false">الافتراضات!$C$7*B38*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)</f>
         <v>2715000</v>
       </c>
-      <c r="D38" s="50" t="n">
+      <c r="D38" s="52" t="n">
         <f aca="false">IFERROR(C38/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$16+الافتراضات!$C$17)),0)</f>
         <v>0.187370600414079</v>
       </c>
@@ -3978,23 +4395,23 @@
         <f aca="false">الافتراضات!$C$7*B38*(1-الافتراضات!$C$30-الافتراضات!$C$31)-الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)</f>
         <v>3405000</v>
       </c>
-      <c r="F38" s="50" t="n">
+      <c r="F38" s="52" t="n">
         <f aca="false">IFERROR(E38/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)),0)</f>
         <v>0.246739130434783</v>
       </c>
-      <c r="G38" s="50" t="n">
+      <c r="G38" s="52" t="n">
         <f aca="false">IFERROR((الافتراضات!$C$7*B38*(1-الافتراضات!$C$30-الافتراضات!$C$31)/(الافتراضات!$C$7*الافتراضات!$C$8*(1+الافتراضات!$C$17)))^(1/الافتراضات!$C$28)-1,0)</f>
         <v>0.116574731236017</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="2" t="s">
-        <v>242</v>
+        <v>261</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="3" t="s">
-        <v>243</v>
+        <v>262</v>
       </c>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
@@ -4005,7 +4422,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="4" t="s">
-        <v>244</v>
+        <v>263</v>
       </c>
       <c r="C42" s="28" t="n">
         <f aca="false">الافتراضات!$C$7*الافتراضات!$C$33</f>
@@ -4014,7 +4431,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="4" t="s">
-        <v>245</v>
+        <v>264</v>
       </c>
       <c r="C43" s="28" t="n">
         <f aca="false">C42*الافتراضات!$C$34</f>
@@ -4023,7 +4440,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="15" t="s">
-        <v>246</v>
+        <v>265</v>
       </c>
       <c r="C44" s="28" t="n">
         <f aca="false">C43*(1-الافتراضات!$C$35)</f>
@@ -4032,7 +4449,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="4" t="s">
-        <v>247</v>
+        <v>266</v>
       </c>
       <c r="C45" s="47" t="n">
         <f aca="false">IFERROR(C42/C5,0)</f>
@@ -4041,7 +4458,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="15" t="s">
-        <v>248</v>
+        <v>267</v>
       </c>
       <c r="C46" s="47" t="n">
         <f aca="false">IFERROR(C44/C7,0)</f>
@@ -4050,11 +4467,11 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="C47" s="51" t="n">
+        <v>268</v>
+      </c>
+      <c r="C47" s="53" t="n">
         <f aca="false">IFERROR(C42/C9,0)</f>
-        <v>0.0576923076923077</v>
+        <v>0.0564853556485356</v>
       </c>
     </row>
   </sheetData>

</xml_diff>